<commit_message>
Intègre le fichier des paiements exécutés (diminution des besoins)
Chaque paiement est imputé sur les lignes de besoin du bénéficiaire (nom,
sinon nature de l'audit PICI Projets), des plus anciennes aux plus récentes,
et retiré du solde du compte débité ; imputation modifiable dans le HTML ;
nouvelle feuille « Paiements exécutés » ; pas de double comptage à la
réimportation. Libellé « (v10) » retiré de l'audit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NEhkcxCB327Mdpf33KqYQU
</commit_message>
<xml_diff>
--- a/Reporting_Hebdo_CIV_30-09-2026.xlsx
+++ b/Reporting_Hebdo_CIV_30-09-2026.xlsx
@@ -11,14 +11,15 @@
     <sheet sheetId="5" name="Position CI 30-09" state="visible" r:id="rId8"/>
     <sheet sheetId="6" name="Contrôles" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Comparaison RCI" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Méthode &amp; sources" state="visible" r:id="rId11"/>
+    <sheet sheetId="8" name="Paiements exécutés" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Méthode &amp; sources" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2760" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2817" uniqueCount="676">
   <si>
     <t>Reporting Cash Hebdomadaire – Centralisation Côte d'Ivoire</t>
   </si>
@@ -566,15 +567,15 @@
     <t>TERASSON – ECO</t>
   </si>
   <si>
+    <t>PICI – STB</t>
+  </si>
+  <si>
+    <t>PICI – SG</t>
+  </si>
+  <si>
     <t>PICI – ECO</t>
   </si>
   <si>
-    <t>PICI – STB</t>
-  </si>
-  <si>
-    <t>PICI – SG</t>
-  </si>
-  <si>
     <t>SCI FIRST – STB</t>
   </si>
   <si>
@@ -1016,6 +1017,9 @@
     <t>02 GROS ŒUVRE &amp; INSTALLATION DE CHANTIER</t>
   </si>
   <si>
+    <t>07/10/2026</t>
+  </si>
+  <si>
     <t>BCC 0023</t>
   </si>
   <si>
@@ -1691,6 +1695,9 @@
     <t>Reporting modifié : 3 ligne(s) changée(s) de semaine – SCO AO SALAIRE NDF 6,3 M S1→S3, SCO AO SALAIRE NDF 6,3 M S1→S3, SCO AO SALAIRE SEPTEMBRE 11,6 M S1→S3.</t>
   </si>
   <si>
+    <t>Paiements exécutés : 4 paiement(s), 704,7 M ; 704,7 M imputés sur le besoin S1 à S5, déduits du solde des comptes débités.</t>
+  </si>
+  <si>
     <t>Comparaison avec la présentation RCI (Laureen) – mêmes sources, M FCFA</t>
   </si>
   <si>
@@ -1721,6 +1728,9 @@
     <t>Explication</t>
   </si>
   <si>
+    <t>Même besoin · Trésorerie : -704,7 (comptes « Dédié paiement Projet SCO » ou comptes non classés en fonctionnement)</t>
+  </si>
+  <si>
     <t>Même besoin</t>
   </si>
   <si>
@@ -1826,6 +1836,84 @@
     <t>• Comptes indisponibles exclus de la position du reporting : STANBIC-FIRST _ Debt Service, STANBIC-FIRST_LL, STANBIC-FIRST_Disbursement, BNI-RIVIERA(Augmentation), BNI-RIVIERA(DSRA) / Placement (1 195,6 M). La présentation RCI exclut aussi ces fonds (DSR, augmentation, LL, disbursement).</t>
   </si>
   <si>
+    <t>Paiements exécutés depuis la position – diminution des besoins</t>
+  </si>
+  <si>
+    <t>Montant imputé : déduit du reste à payer des lignes indiquées (feuilles de détail, colonnes « Payé »). Déduit du solde = O : montant retiré du solde du compte débité dans la position.</t>
+  </si>
+  <si>
+    <t>Réf.</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Compte débité</t>
+  </si>
+  <si>
+    <t>Bénéficiaire</t>
+  </si>
+  <si>
+    <t>Projet</t>
+  </si>
+  <si>
+    <t>Montant payé FCFA</t>
+  </si>
+  <si>
+    <t>Imputé sur</t>
+  </si>
+  <si>
+    <t>Répartition</t>
+  </si>
+  <si>
+    <t>Imputé S1 à S5 FCFA</t>
+  </si>
+  <si>
+    <t>Non imputé / hors horizon FCFA</t>
+  </si>
+  <si>
+    <t>Déduit du solde</t>
+  </si>
+  <si>
+    <t>PX|ECOBANK-PICI|TGCC|07/10/2026|19324742|0</t>
+  </si>
+  <si>
+    <t>TGCC</t>
+  </si>
+  <si>
+    <t>NOTRE PÈRE</t>
+  </si>
+  <si>
+    <t>BCC 0017 02 GROS ŒUVRE &amp; INSTALLATION DE CHANTIER</t>
+  </si>
+  <si>
+    <t>S1 19,3 M</t>
+  </si>
+  <si>
+    <t>PX|ECOBANK-PICI|TGCC|07/10/2026|629862023|1</t>
+  </si>
+  <si>
+    <t>S1 373,4 M ; S2 256,5 M</t>
+  </si>
+  <si>
+    <t>PX|ECOBANK-PICI|TGCC|07/10/2026|52769692|2</t>
+  </si>
+  <si>
+    <t>S2 52,8 M</t>
+  </si>
+  <si>
+    <t>PX|ECOBANK-PICI|HORECAF|07/10/2026|2709103|3</t>
+  </si>
+  <si>
+    <t>HORECAF</t>
+  </si>
+  <si>
+    <t>HON 0002 BET / MOE / SSI – SCO</t>
+  </si>
+  <si>
+    <t>S1 2,7 M</t>
+  </si>
+  <si>
     <t>Méthode, règles de semaine et sources</t>
   </si>
   <si>
@@ -1887,6 +1975,12 @@
   </si>
   <si>
     <t>Soldes : colonne F de la position (modifiable). Paiements effectués : montant payé et date dans les feuilles de détail (colonnes en jaune) ; seul le reste à payer alimente le reporting. Paiements non prévus : nouvelles lignes dans les feuilles de détail. Le fichier modifié se réimporte dans le générateur HTML pour refaire la présentation.</t>
+  </si>
+  <si>
+    <t>Paiements exécutés</t>
+  </si>
+  <si>
+    <t>2d40a539-PAIEMENTS_EXECUTES.xlsx – chaque paiement est imputé sur les lignes de besoin du bénéficiaire (nom, sinon nature de l'audit PICI Projets), des plus anciennes aux plus récentes ; montant retiré du solde du compte débité s'il est postérieur à la position. Détail dans la feuille « Paiements exécutés ».</t>
   </si>
   <si>
     <t>Comptes indisponibles</t>
@@ -2311,7 +2405,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2496,6 +2590,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -9995,13 +10090,13 @@
         <v>141</v>
       </c>
       <c r="E6" s="77" t="s">
+        <v>142</v>
+      </c>
+      <c r="F6" s="77" t="s">
+        <v>140</v>
+      </c>
+      <c r="G6" s="77" t="s">
         <v>141</v>
-      </c>
-      <c r="F6" s="77" t="s">
-        <v>142</v>
-      </c>
-      <c r="G6" s="77" t="s">
-        <v>140</v>
       </c>
       <c r="H6" s="77" t="s">
         <v>142</v>
@@ -10079,13 +10174,13 @@
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"TERASSON – ECO")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"TERASSON – ECO")</f>
       </c>
       <c r="E7" s="78">
+        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"PICI – STB")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"PICI – STB")</f>
+      </c>
+      <c r="F7" s="78">
+        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"PICI – SG")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"PICI – SG")</f>
+      </c>
+      <c r="G7" s="78">
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"PICI – ECO")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"PICI – ECO")</f>
-      </c>
-      <c r="F7" s="78">
-        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"PICI – STB")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"PICI – STB")</f>
-      </c>
-      <c r="G7" s="78">
-        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"PICI – SG")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"PICI – SG")</f>
       </c>
       <c r="H7" s="78">
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"SCI FIRST – STB")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"SCI FIRST – STB")</f>
@@ -10165,13 +10260,13 @@
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"TERASSON – ECO")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"TERASSON – ECO")</f>
       </c>
       <c r="E8" s="78">
+        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"PICI – STB")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"PICI – STB")</f>
+      </c>
+      <c r="F8" s="78">
+        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"PICI – SG")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"PICI – SG")</f>
+      </c>
+      <c r="G8" s="78">
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"PICI – ECO")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"PICI – ECO")</f>
-      </c>
-      <c r="F8" s="78">
-        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"PICI – STB")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"PICI – STB")</f>
-      </c>
-      <c r="G8" s="78">
-        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"PICI – SG")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"PICI – SG")</f>
       </c>
       <c r="H8" s="78">
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"SCI FIRST – STB")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"SCI FIRST – STB")</f>
@@ -10786,13 +10881,13 @@
         <f>'Position CI 30-09'!F11</f>
       </c>
       <c r="E18" s="84">
+        <f>'Position CI 30-09'!F6</f>
+      </c>
+      <c r="F18" s="84">
+        <f>'Position CI 30-09'!F5</f>
+      </c>
+      <c r="G18" s="84">
         <f>'Position CI 30-09'!F7</f>
-      </c>
-      <c r="F18" s="84">
-        <f>'Position CI 30-09'!F6</f>
-      </c>
-      <c r="G18" s="84">
-        <f>'Position CI 30-09'!F5</f>
       </c>
       <c r="H18" s="84">
         <f>'Position CI 30-09'!F9</f>
@@ -19460,8 +19555,12 @@
       <c r="J8" s="94" t="s">
         <v>213</v>
       </c>
-      <c r="K8" s="95"/>
-      <c r="L8" s="96"/>
+      <c r="K8" s="95">
+        <v>392676186</v>
+      </c>
+      <c r="L8" s="96" t="s">
+        <v>332</v>
+      </c>
       <c r="M8" s="51">
         <f>IF(I8&lt;0,MIN(0,I8+N(K8)),MAX(0,I8-N(K8)))</f>
       </c>
@@ -19480,10 +19579,10 @@
         <v>126</v>
       </c>
       <c r="E9" s="49" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F9" s="49" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G9" s="49" t="s">
         <v>15</v>
@@ -19517,10 +19616,10 @@
         <v>126</v>
       </c>
       <c r="E10" s="49" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="F10" s="49" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="G10" s="49" t="s">
         <v>15</v>
@@ -19554,10 +19653,10 @@
         <v>126</v>
       </c>
       <c r="E11" s="49" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F11" s="49" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G11" s="49" t="s">
         <v>15</v>
@@ -19591,13 +19690,13 @@
         <v>127</v>
       </c>
       <c r="E12" s="49" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F12" s="49" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G12" s="49" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H12" s="51">
         <v>-54903</v>
@@ -19628,13 +19727,13 @@
         <v>127</v>
       </c>
       <c r="E13" s="49" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F13" s="49" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G13" s="49" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H13" s="51">
         <v>-6577</v>
@@ -19665,13 +19764,13 @@
         <v>127</v>
       </c>
       <c r="E14" s="49" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F14" s="49" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G14" s="49" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H14" s="51">
         <v>-82323.18</v>
@@ -19682,8 +19781,12 @@
       <c r="J14" s="94" t="s">
         <v>213</v>
       </c>
-      <c r="K14" s="95"/>
-      <c r="L14" s="96"/>
+      <c r="K14" s="95">
+        <v>2709103</v>
+      </c>
+      <c r="L14" s="96" t="s">
+        <v>332</v>
+      </c>
       <c r="M14" s="51">
         <f>IF(I14&lt;0,MIN(0,I14+N(K14)),MAX(0,I14-N(K14)))</f>
       </c>
@@ -19702,13 +19805,13 @@
         <v>127</v>
       </c>
       <c r="E15" s="49" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F15" s="49" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G15" s="49" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="H15" s="51">
         <v>-8415.19</v>
@@ -19739,13 +19842,13 @@
         <v>127</v>
       </c>
       <c r="E16" s="49" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F16" s="49" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G16" s="49" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H16" s="51">
         <v>-6738.37</v>
@@ -19776,13 +19879,13 @@
         <v>127</v>
       </c>
       <c r="E17" s="49" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F17" s="49" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G17" s="49" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="H17" s="51">
         <v>-105395.81</v>
@@ -19813,13 +19916,13 @@
         <v>127</v>
       </c>
       <c r="E18" s="49" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F18" s="49" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G18" s="49" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="H18" s="51">
         <v>-7000</v>
@@ -19850,10 +19953,10 @@
         <v>127</v>
       </c>
       <c r="E19" s="49" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F19" s="49" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G19" s="49" t="s">
         <v>15</v>
@@ -19887,13 +19990,13 @@
         <v>128</v>
       </c>
       <c r="E20" s="49" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F20" s="49" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G20" s="49" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="H20" s="51">
         <v>-10000</v>
@@ -19924,13 +20027,13 @@
         <v>128</v>
       </c>
       <c r="E21" s="49" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F21" s="49" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G21" s="49" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H21" s="51">
         <v>-1255555.2</v>
@@ -19961,10 +20064,10 @@
         <v>129</v>
       </c>
       <c r="E22" s="49" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F22" s="49" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G22" s="49" t="s">
         <v>15</v>
@@ -19998,10 +20101,10 @@
         <v>129</v>
       </c>
       <c r="E23" s="49" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F23" s="49" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G23" s="49" t="s">
         <v>15</v>
@@ -20041,7 +20144,7 @@
         <v>325</v>
       </c>
       <c r="G24" s="49" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H24" s="51">
         <v>-2000</v>
@@ -20072,13 +20175,13 @@
         <v>125</v>
       </c>
       <c r="E25" s="49" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="F25" s="49" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G25" s="49" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="H25" s="51">
         <v>-6532.01</v>
@@ -20109,10 +20212,10 @@
         <v>125</v>
       </c>
       <c r="E26" s="49" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F26" s="49" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G26" s="49" t="s">
         <v>230</v>
@@ -20146,10 +20249,10 @@
         <v>126</v>
       </c>
       <c r="E27" s="49" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F27" s="49" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="G27" s="49" t="s">
         <v>15</v>
@@ -20183,10 +20286,10 @@
         <v>126</v>
       </c>
       <c r="E28" s="49" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F28" s="49" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G28" s="49" t="s">
         <v>15</v>
@@ -20220,13 +20323,13 @@
         <v>126</v>
       </c>
       <c r="E29" s="49" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F29" s="49" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G29" s="49" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H29" s="51">
         <v>-318222.84</v>
@@ -20257,10 +20360,10 @@
         <v>126</v>
       </c>
       <c r="E30" s="49" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F30" s="49" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G30" s="49" t="s">
         <v>15</v>
@@ -20294,10 +20397,10 @@
         <v>126</v>
       </c>
       <c r="E31" s="49" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F31" s="49" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="G31" s="49" t="s">
         <v>15</v>
@@ -20331,10 +20434,10 @@
         <v>126</v>
       </c>
       <c r="E32" s="49" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F32" s="49" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G32" s="49" t="s">
         <v>15</v>
@@ -20371,7 +20474,7 @@
         <v>330</v>
       </c>
       <c r="F33" s="49" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G33" s="49" t="s">
         <v>15</v>
@@ -20405,10 +20508,10 @@
         <v>126</v>
       </c>
       <c r="E34" s="49" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F34" s="49" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G34" s="49" t="s">
         <v>15</v>
@@ -20442,10 +20545,10 @@
         <v>126</v>
       </c>
       <c r="E35" s="49" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F35" s="49" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G35" s="49" t="s">
         <v>15</v>
@@ -20479,13 +20582,13 @@
         <v>127</v>
       </c>
       <c r="E36" s="49" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F36" s="49" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G36" s="49" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="H36" s="51">
         <v>-59066.62</v>
@@ -20516,13 +20619,13 @@
         <v>127</v>
       </c>
       <c r="E37" s="49" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F37" s="49" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G37" s="49" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="H37" s="51">
         <v>-18066.62</v>
@@ -20553,13 +20656,13 @@
         <v>127</v>
       </c>
       <c r="E38" s="49" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F38" s="49" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G38" s="49" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H38" s="51">
         <v>-41399.65</v>
@@ -20590,13 +20693,13 @@
         <v>127</v>
       </c>
       <c r="E39" s="49" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F39" s="49" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G39" s="49" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H39" s="51">
         <v>-10236.62</v>
@@ -20627,13 +20730,13 @@
         <v>127</v>
       </c>
       <c r="E40" s="49" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F40" s="49" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G40" s="49" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H40" s="51">
         <v>-4428</v>
@@ -20664,13 +20767,13 @@
         <v>127</v>
       </c>
       <c r="E41" s="49" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F41" s="49" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G41" s="49" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="H41" s="51">
         <v>-13438.33</v>
@@ -20701,10 +20804,10 @@
         <v>127</v>
       </c>
       <c r="E42" s="49" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F42" s="49" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G42" s="49" t="s">
         <v>15</v>
@@ -20738,13 +20841,13 @@
         <v>127</v>
       </c>
       <c r="E43" s="49" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F43" s="49" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G43" s="49" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="H43" s="51">
         <v>-8000</v>
@@ -20775,10 +20878,10 @@
         <v>127</v>
       </c>
       <c r="E44" s="49" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F44" s="49" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G44" s="49" t="s">
         <v>15</v>
@@ -20812,13 +20915,13 @@
         <v>128</v>
       </c>
       <c r="E45" s="49" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F45" s="49" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G45" s="49" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="H45" s="51">
         <v>-7000</v>
@@ -20849,10 +20952,10 @@
         <v>129</v>
       </c>
       <c r="E46" s="49" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="F46" s="49" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G46" s="49" t="s">
         <v>15</v>
@@ -20886,10 +20989,10 @@
         <v>129</v>
       </c>
       <c r="E47" s="49" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F47" s="49" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="G47" s="49" t="s">
         <v>15</v>
@@ -20923,10 +21026,10 @@
         <v>129</v>
       </c>
       <c r="E48" s="49" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F48" s="49" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G48" s="49" t="s">
         <v>15</v>
@@ -21014,8 +21117,12 @@
       <c r="J50" s="94" t="s">
         <v>213</v>
       </c>
-      <c r="K50" s="95"/>
-      <c r="L50" s="96"/>
+      <c r="K50" s="95">
+        <v>309280271</v>
+      </c>
+      <c r="L50" s="96" t="s">
+        <v>332</v>
+      </c>
       <c r="M50" s="51">
         <f>IF(I50&lt;0,MIN(0,I50+N(K50)),MAX(0,I50-N(K50)))</f>
       </c>
@@ -21034,10 +21141,10 @@
         <v>126</v>
       </c>
       <c r="E51" s="49" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F51" s="49" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G51" s="49" t="s">
         <v>15</v>
@@ -21071,10 +21178,10 @@
         <v>126</v>
       </c>
       <c r="E52" s="49" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F52" s="49" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G52" s="49" t="s">
         <v>15</v>
@@ -21108,13 +21215,13 @@
         <v>127</v>
       </c>
       <c r="E53" s="49" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F53" s="49" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G53" s="49" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="H53" s="51">
         <v>-4827.48</v>
@@ -21145,13 +21252,13 @@
         <v>127</v>
       </c>
       <c r="E54" s="49" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F54" s="49" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G54" s="49" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="H54" s="51">
         <v>-8253</v>
@@ -21182,10 +21289,10 @@
         <v>127</v>
       </c>
       <c r="E55" s="49" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F55" s="49" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G55" s="49" t="s">
         <v>15</v>
@@ -21219,10 +21326,10 @@
         <v>128</v>
       </c>
       <c r="E56" s="49" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F56" s="49" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G56" s="49" t="s">
         <v>229</v>
@@ -21256,13 +21363,13 @@
         <v>125</v>
       </c>
       <c r="E57" s="49" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F57" s="49" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G57" s="49" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="H57" s="51">
         <v>-22400</v>
@@ -21293,13 +21400,13 @@
         <v>126</v>
       </c>
       <c r="E58" s="49" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F58" s="49" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G58" s="49" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H58" s="51">
         <v>-64093.98</v>
@@ -21330,10 +21437,10 @@
         <v>126</v>
       </c>
       <c r="E59" s="49" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F59" s="49" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G59" s="49" t="s">
         <v>15</v>
@@ -21367,10 +21474,10 @@
         <v>126</v>
       </c>
       <c r="E60" s="49" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F60" s="49" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G60" s="49" t="s">
         <v>15</v>
@@ -21404,10 +21511,10 @@
         <v>126</v>
       </c>
       <c r="E61" s="49" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F61" s="49" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G61" s="49" t="s">
         <v>15</v>
@@ -21441,10 +21548,10 @@
         <v>126</v>
       </c>
       <c r="E62" s="49" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F62" s="49" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G62" s="49" t="s">
         <v>15</v>
@@ -21481,7 +21588,7 @@
         <v>330</v>
       </c>
       <c r="F63" s="49" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G63" s="49" t="s">
         <v>15</v>
@@ -21515,13 +21622,13 @@
         <v>127</v>
       </c>
       <c r="E64" s="49" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F64" s="49" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G64" s="49" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="H64" s="51">
         <v>-6719.33</v>
@@ -21552,10 +21659,10 @@
         <v>127</v>
       </c>
       <c r="E65" s="49" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F65" s="49" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G65" s="49" t="s">
         <v>15</v>
@@ -21589,13 +21696,13 @@
         <v>128</v>
       </c>
       <c r="E66" s="49" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F66" s="49" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G66" s="49" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="H66" s="51">
         <v>-11683</v>
@@ -21626,13 +21733,13 @@
         <v>128</v>
       </c>
       <c r="E67" s="49" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F67" s="49" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G67" s="49" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="H67" s="51">
         <v>-3000</v>
@@ -21663,13 +21770,13 @@
         <v>128</v>
       </c>
       <c r="E68" s="49" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F68" s="49" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G68" s="49" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="H68" s="51">
         <v>-35480</v>
@@ -21700,10 +21807,10 @@
         <v>129</v>
       </c>
       <c r="E69" s="49" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F69" s="49" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G69" s="49" t="s">
         <v>15</v>
@@ -21737,10 +21844,10 @@
         <v>129</v>
       </c>
       <c r="E70" s="49" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F70" s="49" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G70" s="49" t="s">
         <v>15</v>
@@ -21774,13 +21881,13 @@
         <v>127</v>
       </c>
       <c r="E71" s="49" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F71" s="49" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G71" s="49" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H71" s="51">
         <v>-20580.8</v>
@@ -21811,13 +21918,13 @@
         <v>127</v>
       </c>
       <c r="E72" s="49" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F72" s="49" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G72" s="49" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H72" s="51">
         <v>-20699.65</v>
@@ -21836,7 +21943,7 @@
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B73" s="98" t="s">
         <v>70</v>
@@ -21848,10 +21955,10 @@
         <v>126</v>
       </c>
       <c r="E73" s="98" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F73" s="98" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G73" s="98" t="s">
         <v>15</v>
@@ -21873,7 +21980,7 @@
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B74" s="98" t="s">
         <v>70</v>
@@ -21910,7 +22017,7 @@
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B75" s="98" t="s">
         <v>70</v>
@@ -21947,7 +22054,7 @@
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B76" s="98" t="s">
         <v>70</v>
@@ -21959,10 +22066,10 @@
         <v>126</v>
       </c>
       <c r="E76" s="98" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F76" s="98" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G76" s="98" t="s">
         <v>15</v>
@@ -21984,7 +22091,7 @@
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B77" s="98" t="s">
         <v>70</v>
@@ -21996,10 +22103,10 @@
         <v>126</v>
       </c>
       <c r="E77" s="98" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F77" s="98" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G77" s="98" t="s">
         <v>15</v>
@@ -22021,7 +22128,7 @@
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B78" s="98" t="s">
         <v>70</v>
@@ -22033,10 +22140,10 @@
         <v>126</v>
       </c>
       <c r="E78" s="98" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F78" s="98" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G78" s="98" t="s">
         <v>15</v>
@@ -22058,7 +22165,7 @@
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B79" s="98" t="s">
         <v>70</v>
@@ -22070,10 +22177,10 @@
         <v>126</v>
       </c>
       <c r="E79" s="98" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F79" s="98" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G79" s="98" t="s">
         <v>15</v>
@@ -22095,7 +22202,7 @@
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B80" s="98" t="s">
         <v>70</v>
@@ -22107,10 +22214,10 @@
         <v>126</v>
       </c>
       <c r="E80" s="98" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F80" s="98" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G80" s="98" t="s">
         <v>15</v>
@@ -22132,7 +22239,7 @@
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B81" s="98" t="s">
         <v>70</v>
@@ -22144,10 +22251,10 @@
         <v>126</v>
       </c>
       <c r="E81" s="98" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F81" s="98" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G81" s="98" t="s">
         <v>15</v>
@@ -22169,7 +22276,7 @@
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B82" s="98" t="s">
         <v>70</v>
@@ -22181,10 +22288,10 @@
         <v>126</v>
       </c>
       <c r="E82" s="98" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F82" s="98" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G82" s="98" t="s">
         <v>15</v>
@@ -22206,7 +22313,7 @@
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B83" s="98" t="s">
         <v>70</v>
@@ -22218,13 +22325,13 @@
         <v>127</v>
       </c>
       <c r="E83" s="98" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F83" s="98" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G83" s="98" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H83" s="99">
         <v>-6577</v>
@@ -22243,7 +22350,7 @@
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A84" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B84" s="98" t="s">
         <v>70</v>
@@ -22255,13 +22362,13 @@
         <v>127</v>
       </c>
       <c r="E84" s="98" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F84" s="98" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G84" s="98" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H84" s="99">
         <v>-20580.8</v>
@@ -22280,7 +22387,7 @@
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B85" s="98" t="s">
         <v>70</v>
@@ -22292,13 +22399,13 @@
         <v>127</v>
       </c>
       <c r="E85" s="98" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F85" s="98" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G85" s="98" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H85" s="99">
         <v>-4878.37</v>
@@ -22317,7 +22424,7 @@
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A86" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B86" s="98" t="s">
         <v>70</v>
@@ -22329,13 +22436,13 @@
         <v>127</v>
       </c>
       <c r="E86" s="98" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F86" s="98" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G86" s="98" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="H86" s="99">
         <v>-4827.48</v>
@@ -22354,7 +22461,7 @@
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B87" s="98" t="s">
         <v>70</v>
@@ -22366,10 +22473,10 @@
         <v>127</v>
       </c>
       <c r="E87" s="98" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F87" s="98" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G87" s="98" t="s">
         <v>15</v>
@@ -22391,7 +22498,7 @@
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B88" s="98" t="s">
         <v>70</v>
@@ -22403,10 +22510,10 @@
         <v>128</v>
       </c>
       <c r="E88" s="98" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F88" s="98" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G88" s="98" t="s">
         <v>229</v>
@@ -22428,7 +22535,7 @@
     </row>
     <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B89" s="98" t="s">
         <v>70</v>
@@ -22440,13 +22547,13 @@
         <v>128</v>
       </c>
       <c r="E89" s="98" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F89" s="98" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G89" s="98" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="H89" s="99">
         <v>-42996.69</v>
@@ -22465,7 +22572,7 @@
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B90" s="98" t="s">
         <v>70</v>
@@ -22474,13 +22581,13 @@
         <v>33</v>
       </c>
       <c r="D90" s="98" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E90" s="98" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F90" s="98" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G90" s="98" t="s">
         <v>15</v>
@@ -22502,7 +22609,7 @@
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B91" s="98" t="s">
         <v>70</v>
@@ -22511,13 +22618,13 @@
         <v>33</v>
       </c>
       <c r="D91" s="98" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E91" s="98" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F91" s="98" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="G91" s="98" t="s">
         <v>15</v>
@@ -22539,7 +22646,7 @@
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B92" s="98" t="s">
         <v>70</v>
@@ -22551,13 +22658,13 @@
         <v>129</v>
       </c>
       <c r="E92" s="98" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F92" s="98" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="G92" s="98" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="H92" s="99">
         <v>-289547.42</v>
@@ -22576,7 +22683,7 @@
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B93" s="98" t="s">
         <v>70</v>
@@ -22588,13 +22695,13 @@
         <v>129</v>
       </c>
       <c r="E93" s="98" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F93" s="98" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G93" s="98" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="H93" s="99">
         <v>-44236.41</v>
@@ -22613,7 +22720,7 @@
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A94" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B94" s="98" t="s">
         <v>67</v>
@@ -22625,10 +22732,10 @@
         <v>126</v>
       </c>
       <c r="E94" s="98" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="F94" s="98" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="G94" s="98" t="s">
         <v>15</v>
@@ -22650,7 +22757,7 @@
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A95" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B95" s="98" t="s">
         <v>67</v>
@@ -22662,13 +22769,13 @@
         <v>126</v>
       </c>
       <c r="E95" s="98" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="F95" s="98" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="G95" s="98" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="H95" s="99">
         <v>-87897.35</v>
@@ -22687,7 +22794,7 @@
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A96" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B96" s="98" t="s">
         <v>67</v>
@@ -22699,10 +22806,10 @@
         <v>126</v>
       </c>
       <c r="E96" s="98" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F96" s="98" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G96" s="98" t="s">
         <v>15</v>
@@ -22724,7 +22831,7 @@
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A97" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B97" s="98" t="s">
         <v>67</v>
@@ -22736,10 +22843,10 @@
         <v>126</v>
       </c>
       <c r="E97" s="98" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F97" s="98" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G97" s="98" t="s">
         <v>15</v>
@@ -22761,7 +22868,7 @@
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B98" s="98" t="s">
         <v>67</v>
@@ -22773,13 +22880,13 @@
         <v>127</v>
       </c>
       <c r="E98" s="98" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="F98" s="98" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="G98" s="98" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="H98" s="99">
         <v>-18066.62</v>
@@ -22798,7 +22905,7 @@
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B99" s="98" t="s">
         <v>67</v>
@@ -22810,13 +22917,13 @@
         <v>127</v>
       </c>
       <c r="E99" s="98" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F99" s="98" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G99" s="98" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H99" s="99">
         <v>-20699.65</v>
@@ -22835,7 +22942,7 @@
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B100" s="98" t="s">
         <v>67</v>
@@ -22847,13 +22954,13 @@
         <v>127</v>
       </c>
       <c r="E100" s="98" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F100" s="98" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G100" s="98" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="H100" s="99">
         <v>-6719.33</v>
@@ -22872,7 +22979,7 @@
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B101" s="98" t="s">
         <v>67</v>
@@ -22884,13 +22991,13 @@
         <v>127</v>
       </c>
       <c r="E101" s="98" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F101" s="98" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G101" s="98" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="H101" s="99">
         <v>-10000</v>
@@ -22909,7 +23016,7 @@
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B102" s="98" t="s">
         <v>67</v>
@@ -22921,10 +23028,10 @@
         <v>127</v>
       </c>
       <c r="E102" s="98" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="F102" s="98" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="G102" s="98" t="s">
         <v>15</v>
@@ -22946,7 +23053,7 @@
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B103" s="98" t="s">
         <v>67</v>
@@ -22958,13 +23065,13 @@
         <v>128</v>
       </c>
       <c r="E103" s="98" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F103" s="98" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G103" s="98" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H103" s="99">
         <v>-8600</v>
@@ -22983,7 +23090,7 @@
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B104" s="98" t="s">
         <v>67</v>
@@ -22995,13 +23102,13 @@
         <v>128</v>
       </c>
       <c r="E104" s="98" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F104" s="98" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G104" s="98" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="H104" s="99">
         <v>-10394.35</v>
@@ -23020,7 +23127,7 @@
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" s="97" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B105" s="98" t="s">
         <v>67</v>
@@ -23032,13 +23139,13 @@
         <v>128</v>
       </c>
       <c r="E105" s="98" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F105" s="98" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G105" s="98" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="H105" s="99">
         <v>-8000</v>
@@ -23066,13 +23173,13 @@
         <v>33</v>
       </c>
       <c r="D106" s="98" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E106" s="98" t="s">
         <v>15</v>
       </c>
       <c r="F106" s="98" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="G106" s="98" t="s">
         <v>15</v>
@@ -23103,13 +23210,13 @@
         <v>36</v>
       </c>
       <c r="D107" s="98" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E107" s="98" t="s">
         <v>15</v>
       </c>
       <c r="F107" s="98" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G107" s="98" t="s">
         <v>15</v>
@@ -25913,12 +26020,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="74" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -25926,34 +26033,34 @@
         <v>97</v>
       </c>
       <c r="B4" s="93" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="C4" s="93" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D4" s="93" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="93" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F4" s="93" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G4" s="93" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="H4" s="93" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="I4" s="93" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J4" s="93" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K4" s="93" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -25961,16 +26068,16 @@
         <v>22</v>
       </c>
       <c r="B5" s="49" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C5" s="49" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D5" s="49" t="s">
         <v>25</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F5" s="95">
         <v>3580753</v>
@@ -25982,7 +26089,7 @@
         <v>22</v>
       </c>
       <c r="I5" s="49" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J5" s="51">
         <v>3580753</v>
@@ -25996,16 +26103,16 @@
         <v>22</v>
       </c>
       <c r="B6" s="49" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C6" s="49" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D6" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E6" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F6" s="95">
         <v>24751125</v>
@@ -26017,7 +26124,7 @@
         <v>22</v>
       </c>
       <c r="I6" s="49" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="J6" s="51">
         <v>24751125</v>
@@ -26031,19 +26138,19 @@
         <v>22</v>
       </c>
       <c r="B7" s="49" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C7" s="49" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D7" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E7" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F7" s="95">
-        <v>368235073</v>
+        <v>-336430487</v>
       </c>
       <c r="G7" s="51">
         <f>F7/'Reporting Hebdo'!$E$3</f>
@@ -26052,7 +26159,7 @@
         <v>22</v>
       </c>
       <c r="I7" s="49" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J7" s="51">
         <v>368235073</v>
@@ -26066,16 +26173,16 @@
         <v>29</v>
       </c>
       <c r="B8" s="49" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C8" s="49" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D8" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E8" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F8" s="95">
         <v>8429337</v>
@@ -26087,7 +26194,7 @@
         <v>29</v>
       </c>
       <c r="I8" s="49" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="J8" s="51">
         <v>8429337</v>
@@ -26101,16 +26208,16 @@
         <v>29</v>
       </c>
       <c r="B9" s="49" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C9" s="49" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D9" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E9" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F9" s="95">
         <v>227694317</v>
@@ -26122,7 +26229,7 @@
         <v>29</v>
       </c>
       <c r="I9" s="49" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="J9" s="51">
         <v>227694317</v>
@@ -26136,16 +26243,16 @@
         <v>33</v>
       </c>
       <c r="B10" s="49" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C10" s="49" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D10" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E10" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F10" s="95">
         <v>58193022</v>
@@ -26157,7 +26264,7 @@
         <v>33</v>
       </c>
       <c r="I10" s="49" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J10" s="51">
         <v>58193022</v>
@@ -26171,16 +26278,16 @@
         <v>33</v>
       </c>
       <c r="B11" s="49" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C11" s="49" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D11" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E11" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F11" s="95">
         <v>62000</v>
@@ -26192,7 +26299,7 @@
         <v>33</v>
       </c>
       <c r="I11" s="49" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="J11" s="51">
         <v>62000</v>
@@ -26206,16 +26313,16 @@
         <v>36</v>
       </c>
       <c r="B12" s="49" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C12" s="49" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D12" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E12" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F12" s="95">
         <v>1473216</v>
@@ -26227,7 +26334,7 @@
         <v>36</v>
       </c>
       <c r="I12" s="49" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="J12" s="51">
         <v>1473216</v>
@@ -26241,16 +26348,16 @@
         <v>36</v>
       </c>
       <c r="B13" s="49" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C13" s="49" t="s">
         <v>65</v>
       </c>
       <c r="D13" s="49" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="E13" s="49" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F13" s="95">
         <v>1771977229</v>
@@ -26262,7 +26369,7 @@
         <v>64</v>
       </c>
       <c r="I13" s="49" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="J13" s="51">
         <v>1771977229</v>
@@ -26276,16 +26383,16 @@
         <v>39</v>
       </c>
       <c r="B14" s="49" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="C14" s="49" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D14" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E14" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F14" s="95">
         <v>897338</v>
@@ -26297,7 +26404,7 @@
         <v>39</v>
       </c>
       <c r="I14" s="49" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="J14" s="51">
         <v>897338</v>
@@ -26311,16 +26418,16 @@
         <v>39</v>
       </c>
       <c r="B15" s="49" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C15" s="49" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D15" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E15" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F15" s="95">
         <v>5375161</v>
@@ -26332,7 +26439,7 @@
         <v>39</v>
       </c>
       <c r="I15" s="49" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="J15" s="51">
         <v>5375161</v>
@@ -26346,16 +26453,16 @@
         <v>39</v>
       </c>
       <c r="B16" s="49" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C16" s="49" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D16" s="49" t="s">
         <v>43</v>
       </c>
       <c r="E16" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F16" s="95">
         <v>22569647</v>
@@ -26367,7 +26474,7 @@
         <v>39</v>
       </c>
       <c r="I16" s="49" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="J16" s="51">
         <v>22569647</v>
@@ -26381,16 +26488,16 @@
         <v>39</v>
       </c>
       <c r="B17" s="49" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C17" s="49" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="D17" s="49" t="s">
         <v>43</v>
       </c>
       <c r="E17" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F17" s="95">
         <v>227288</v>
@@ -26402,7 +26509,7 @@
         <v>39</v>
       </c>
       <c r="I17" s="49" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="J17" s="51">
         <v>227288</v>
@@ -26416,16 +26523,16 @@
         <v>39</v>
       </c>
       <c r="B18" s="49" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C18" s="49" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="D18" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E18" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F18" s="95">
         <v>62000</v>
@@ -26437,7 +26544,7 @@
         <v>39</v>
       </c>
       <c r="I18" s="49" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="J18" s="51">
         <v>62000</v>
@@ -26451,16 +26558,16 @@
         <v>46</v>
       </c>
       <c r="B19" s="49" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C19" s="49" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D19" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E19" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F19" s="95">
         <v>35011732</v>
@@ -26472,7 +26579,7 @@
         <v>46</v>
       </c>
       <c r="I19" s="49" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="J19" s="51">
         <v>35011732</v>
@@ -26486,16 +26593,16 @@
         <v>46</v>
       </c>
       <c r="B20" s="49" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C20" s="49" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D20" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E20" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F20" s="95">
         <v>62000</v>
@@ -26507,7 +26614,7 @@
         <v>46</v>
       </c>
       <c r="I20" s="49" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="J20" s="51">
         <v>62000</v>
@@ -26521,16 +26628,16 @@
         <v>50</v>
       </c>
       <c r="B21" s="49" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C21" s="49" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="D21" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E21" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F21" s="95">
         <v>-74342</v>
@@ -26542,7 +26649,7 @@
         <v>50</v>
       </c>
       <c r="I21" s="49" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="J21" s="51">
         <v>-74342</v>
@@ -26556,16 +26663,16 @@
         <v>50</v>
       </c>
       <c r="B22" s="49" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C22" s="49" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D22" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E22" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F22" s="95">
         <v>62000</v>
@@ -26577,7 +26684,7 @@
         <v>50</v>
       </c>
       <c r="I22" s="49" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="J22" s="51">
         <v>62000</v>
@@ -26591,16 +26698,16 @@
         <v>53</v>
       </c>
       <c r="B23" s="49" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C23" s="49" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="D23" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E23" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F23" s="95">
         <v>11670561</v>
@@ -26612,7 +26719,7 @@
         <v>53</v>
       </c>
       <c r="I23" s="49" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="J23" s="51">
         <v>11670561</v>
@@ -26626,16 +26733,16 @@
         <v>53</v>
       </c>
       <c r="B24" s="49" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="C24" s="49" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D24" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E24" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F24" s="95">
         <v>36000</v>
@@ -26647,7 +26754,7 @@
         <v>53</v>
       </c>
       <c r="I24" s="49" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="J24" s="51">
         <v>36000</v>
@@ -26670,7 +26777,7 @@
         <v>27</v>
       </c>
       <c r="E25" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F25" s="95">
         <v>58000</v>
@@ -26682,7 +26789,7 @@
         <v>53</v>
       </c>
       <c r="I25" s="49" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="J25" s="51">
         <v>58000</v>
@@ -26699,13 +26806,13 @@
         <v>149</v>
       </c>
       <c r="C26" s="49" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="D26" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E26" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F26" s="95">
         <v>2751880</v>
@@ -26717,7 +26824,7 @@
         <v>57</v>
       </c>
       <c r="I26" s="49" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="J26" s="51">
         <v>2751880</v>
@@ -26731,16 +26838,16 @@
         <v>59</v>
       </c>
       <c r="B27" s="49" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="C27" s="49" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D27" s="49" t="s">
         <v>27</v>
       </c>
       <c r="E27" s="49" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="F27" s="95">
         <v>6062002</v>
@@ -26752,7 +26859,7 @@
         <v>59</v>
       </c>
       <c r="I27" s="49" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="J27" s="51">
         <v>6062002</v>
@@ -26766,16 +26873,16 @@
         <v>36</v>
       </c>
       <c r="B28" s="49" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C28" s="49" t="s">
         <v>68</v>
       </c>
       <c r="D28" s="49" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E28" s="49" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F28" s="95">
         <v>2643139493</v>
@@ -26787,7 +26894,7 @@
         <v>67</v>
       </c>
       <c r="I28" s="49" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="J28" s="51">
         <v>2643139493</v>
@@ -26801,16 +26908,16 @@
         <v>33</v>
       </c>
       <c r="B29" s="49" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C29" s="49" t="s">
         <v>71</v>
       </c>
       <c r="D29" s="49" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E29" s="49" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F29" s="95">
         <v>1481904490</v>
@@ -26822,7 +26929,7 @@
         <v>70</v>
       </c>
       <c r="I29" s="49" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="J29" s="51">
         <v>1481904490</v>
@@ -26845,7 +26952,7 @@
         <v>79</v>
       </c>
       <c r="E30" s="49" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="F30" s="95">
         <v>76268390</v>
@@ -26857,7 +26964,7 @@
         <v>72</v>
       </c>
       <c r="I30" s="49" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="J30" s="51">
         <v>76268390</v>
@@ -26868,7 +26975,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="104" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="F31" s="105">
         <f>SUM(F5:F30)</f>
@@ -26879,7 +26986,7 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -26887,7 +26994,7 @@
         <v>29</v>
       </c>
       <c r="B35" s="98" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C35" s="98" t="s">
         <v>78</v>
@@ -26896,7 +27003,7 @@
         <v>79</v>
       </c>
       <c r="E35" s="98" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F35" s="99">
         <v>350727089</v>
@@ -26908,7 +27015,7 @@
         <v>15</v>
       </c>
       <c r="I35" s="98" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="J35" s="98">
         <v>350727089</v>
@@ -26919,7 +27026,7 @@
         <v>29</v>
       </c>
       <c r="B36" s="98" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C36" s="98" t="s">
         <v>80</v>
@@ -26928,7 +27035,7 @@
         <v>79</v>
       </c>
       <c r="E36" s="98" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F36" s="99">
         <v>42500000</v>
@@ -26940,7 +27047,7 @@
         <v>15</v>
       </c>
       <c r="I36" s="98" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="J36" s="98">
         <v>42500000</v>
@@ -26951,7 +27058,7 @@
         <v>29</v>
       </c>
       <c r="B37" s="98" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="C37" s="98" t="s">
         <v>81</v>
@@ -26960,7 +27067,7 @@
         <v>79</v>
       </c>
       <c r="E37" s="98" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F37" s="99">
         <v>26289357</v>
@@ -26972,7 +27079,7 @@
         <v>15</v>
       </c>
       <c r="I37" s="98" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="J37" s="98">
         <v>26289357</v>
@@ -26983,7 +27090,7 @@
         <v>36</v>
       </c>
       <c r="B38" s="98" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C38" s="98" t="s">
         <v>82</v>
@@ -26992,7 +27099,7 @@
         <v>79</v>
       </c>
       <c r="E38" s="98" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F38" s="99">
         <v>0</v>
@@ -27004,7 +27111,7 @@
         <v>15</v>
       </c>
       <c r="I38" s="98" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="J38" s="98">
         <v>0</v>
@@ -27015,7 +27122,7 @@
         <v>36</v>
       </c>
       <c r="B39" s="98" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="C39" s="98" t="s">
         <v>83</v>
@@ -27024,7 +27131,7 @@
         <v>79</v>
       </c>
       <c r="E39" s="98" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="F39" s="99">
         <v>776110097</v>
@@ -27036,7 +27143,7 @@
         <v>15</v>
       </c>
       <c r="I39" s="98" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="J39" s="98">
         <v>776110097</v>
@@ -27044,7 +27151,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="106" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F40" s="107">
         <f>SUM(F35:F39)</f>
@@ -27058,7 +27165,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="70" customWidth="1"/>
@@ -27070,34 +27177,34 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="93" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B4" s="93" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C4" s="93" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="D4" s="93" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E4" s="93" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="49" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B5" s="51">
         <f>'Reporting Hebdo'!M52</f>
@@ -27109,12 +27216,12 @@
         <f>B5-C5</f>
       </c>
       <c r="E5" s="49" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -27122,16 +27229,16 @@
         <v>97</v>
       </c>
       <c r="B8" s="93" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="C8" s="93" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D8" s="93" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E8" s="93" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -27148,7 +27255,7 @@
         <f>B9-C9</f>
       </c>
       <c r="E9" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -27165,7 +27272,7 @@
         <f>B10-C10</f>
       </c>
       <c r="E10" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -27182,7 +27289,7 @@
         <f>B11-C11</f>
       </c>
       <c r="E11" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -27199,7 +27306,7 @@
         <f>B12-C12</f>
       </c>
       <c r="E12" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -27216,7 +27323,7 @@
         <f>B13-C13</f>
       </c>
       <c r="E13" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -27233,7 +27340,7 @@
         <f>B14-C14</f>
       </c>
       <c r="E14" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -27250,7 +27357,7 @@
         <f>B15-C15</f>
       </c>
       <c r="E15" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -27267,7 +27374,7 @@
         <f>B16-C16</f>
       </c>
       <c r="E16" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -27284,34 +27391,34 @@
         <f>B17-C17</f>
       </c>
       <c r="E17" s="49" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="93" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B20" s="93" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="C20" s="93" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D20" s="93" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E20" s="93" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="49" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B21" s="51">
         <f>-SUMIFS('Détail projets &amp; dettes'!$H$5:$H$500,'Détail projets &amp; dettes'!$C$5:$C$500,"RIVIERA",'Détail projets &amp; dettes'!$J$5:$J$500,"O",'Détail projets &amp; dettes'!$A$5:$A$500,"S*")</f>
@@ -27323,12 +27430,12 @@
         <f>B21-C21</f>
       </c>
       <c r="E21" s="49" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="49" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B22" s="51">
         <f>-SUMIFS('Détail projets &amp; dettes'!$H$5:$H$500,'Détail projets &amp; dettes'!$C$5:$C$500,"TERASSON",'Détail projets &amp; dettes'!$J$5:$J$500,"O",'Détail projets &amp; dettes'!$A$5:$A$500,"S*")</f>
@@ -27340,34 +27447,34 @@
         <f>B22-C22</f>
       </c>
       <c r="E22" s="49" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="93" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B25" s="93" t="s">
         <v>173</v>
       </c>
       <c r="C25" s="93" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="D25" s="93" t="s">
         <v>15</v>
       </c>
       <c r="E25" s="93" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="49" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B26" s="51">
         <v>-13254203304</v>
@@ -27379,12 +27486,12 @@
         <v>15</v>
       </c>
       <c r="E26" s="49" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B27" s="51">
         <v>-1715342550</v>
@@ -27396,12 +27503,12 @@
         <v>15</v>
       </c>
       <c r="E27" s="49" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="49" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B28" s="51">
         <v>6113285</v>
@@ -27413,12 +27520,12 @@
         <v>15</v>
       </c>
       <c r="E28" s="49" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="49" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B29" s="51">
         <v>-220402934</v>
@@ -27430,17 +27537,22 @@
         <v>15</v>
       </c>
       <c r="E29" s="49" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="89" t="s">
-        <v>556</v>
+        <v>557</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="89" t="s">
+        <v>558</v>
       </c>
     </row>
   </sheetData>
@@ -27463,12 +27575,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -27476,31 +27588,31 @@
         <v>97</v>
       </c>
       <c r="B4" s="93" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="C4" s="93" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="D4" s="93" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E4" s="93" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="F4" s="93" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="G4" s="93" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="H4" s="93" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="I4" s="93" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="J4" s="93" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -27520,19 +27632,19 @@
         <v>396.566951</v>
       </c>
       <c r="F5" s="110">
-        <v>396.566951</v>
+        <v>-308.098609</v>
       </c>
       <c r="G5" s="110">
         <v>99.98971200000005</v>
       </c>
       <c r="H5" s="110">
-        <v>99.98971200000005</v>
+        <v>-604.675848</v>
       </c>
       <c r="I5" s="110">
-        <v>0</v>
+        <v>-704.66556</v>
       </c>
       <c r="J5" s="111" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -27564,7 +27676,7 @@
         <v>-5.684341886080802e-14</v>
       </c>
       <c r="J6" s="111" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -27596,7 +27708,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="111" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -27628,7 +27740,7 @@
         <v>1.4210854715202004e-14</v>
       </c>
       <c r="J8" s="111" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -27654,7 +27766,7 @@
         <v>-176.007224</v>
       </c>
       <c r="J9" s="111" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -27686,7 +27798,7 @@
         <v>2.842170943040401e-14</v>
       </c>
       <c r="J10" s="111" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -27718,7 +27830,7 @@
         <v>0</v>
       </c>
       <c r="J11" s="111" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -27750,7 +27862,7 @@
         <v>-1.4210854715202004e-14</v>
       </c>
       <c r="J12" s="111" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -27776,7 +27888,7 @@
         <v>2.75188</v>
       </c>
       <c r="J13" s="111" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -27808,7 +27920,7 @@
         <v>-1.7763568394002505e-15</v>
       </c>
       <c r="J14" s="111" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -27840,7 +27952,7 @@
         <v>-1.4210854715202004e-14</v>
       </c>
       <c r="J15" s="111" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -27860,16 +27972,16 @@
         <v>745.306796</v>
       </c>
       <c r="F16" s="112">
-        <v>777.19011</v>
+        <v>72.52454999999998</v>
       </c>
       <c r="G16" s="112">
         <v>-693.5213609829399</v>
       </c>
       <c r="H16" s="112">
-        <v>-866.7767049829399</v>
+        <v>-1571.4422649829398</v>
       </c>
       <c r="I16" s="112">
-        <v>-173.2553440000001</v>
+        <v>-877.9209040000001</v>
       </c>
       <c r="J16" s="54" t="s">
         <v>15</v>
@@ -27877,29 +27989,29 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="93" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B19" s="93" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="C19" s="93" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="D19" s="93" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E19" s="93" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="49" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B20" s="110">
         <v>244.99626199999997</v>
@@ -27911,12 +28023,12 @@
         <v>0</v>
       </c>
       <c r="E20" s="49" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="49" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="B21" s="110">
         <v>637.405803</v>
@@ -27928,12 +28040,12 @@
         <v>0</v>
       </c>
       <c r="E21" s="49" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="49" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B22" s="110">
         <v>152.070689</v>
@@ -27945,7 +28057,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="49" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -27962,12 +28074,12 @@
         <v>0</v>
       </c>
       <c r="E23" s="49" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="49" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="B24" s="110">
         <v>448.13497721294</v>
@@ -27979,12 +28091,12 @@
         <v>0</v>
       </c>
       <c r="E24" s="49" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="49" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="B25" s="110">
         <v>129.56826523</v>
@@ -27996,12 +28108,12 @@
         <v>-2.842170943040401e-14</v>
       </c>
       <c r="E25" s="49" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="49" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="B26" s="110">
         <v>0</v>
@@ -28013,29 +28125,29 @@
         <v>208.73865799999996</v>
       </c>
       <c r="E26" s="49" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="93" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B29" s="93" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="C29" s="93" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -28052,12 +28164,12 @@
         <v>4.547473508864641e-13</v>
       </c>
       <c r="E30" s="54" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="49" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="B31" s="110">
         <v>91.2699500964329</v>
@@ -28069,12 +28181,12 @@
         <v>0</v>
       </c>
       <c r="E31" s="49" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="49" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="B32" s="110">
         <v>1976.5850833750312</v>
@@ -28086,12 +28198,12 @@
         <v>0</v>
       </c>
       <c r="E32" s="49" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="49" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B33" s="110">
         <v>1267.9055957833798</v>
@@ -28103,12 +28215,12 @@
         <v>2.2737367544323206e-13</v>
       </c>
       <c r="E33" s="49" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="49" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="B34" s="110">
         <v>455.07613148087546</v>
@@ -28120,12 +28232,12 @@
         <v>-1.1368683772161603e-13</v>
       </c>
       <c r="E34" s="49" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="49" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B35" s="110">
         <v>2643.139493</v>
@@ -28137,7 +28249,7 @@
         <v>0</v>
       </c>
       <c r="E35" s="49" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -28148,18 +28260,18 @@
         <v>3926.313997203903</v>
       </c>
       <c r="C36" s="112">
-        <v>3926.313997203903</v>
+        <v>3221.648437203903</v>
       </c>
       <c r="D36" s="112">
-        <v>0</v>
+        <v>-704.6655599999999</v>
       </c>
       <c r="E36" s="54" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="49" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="B37" s="110">
         <v>116.22847414168119</v>
@@ -28171,12 +28283,12 @@
         <v>1.4210854715202004e-14</v>
       </c>
       <c r="E37" s="49" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="49" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="B38" s="110">
         <v>2197.7624460785723</v>
@@ -28188,12 +28300,12 @@
         <v>0</v>
       </c>
       <c r="E38" s="49" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="49" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="B39" s="110">
         <v>490.0631747136942</v>
@@ -28205,12 +28317,12 @@
         <v>0</v>
       </c>
       <c r="E39" s="49" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="49" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="B40" s="110">
         <v>1238.4883764116369</v>
@@ -28222,12 +28334,12 @@
         <v>-2.2737367544323206e-13</v>
       </c>
       <c r="E40" s="49" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="49" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="B41" s="110">
         <v>1481.90449</v>
@@ -28239,17 +28351,17 @@
         <v>0</v>
       </c>
       <c r="E41" s="49" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="113" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="B44" s="113"/>
       <c r="C44" s="113"/>
@@ -28263,7 +28375,7 @@
     </row>
     <row r="45" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="113" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="B45" s="113"/>
       <c r="C45" s="113"/>
@@ -28277,7 +28389,7 @@
     </row>
     <row r="46" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="113" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="B46" s="113"/>
       <c r="C46" s="113"/>
@@ -28291,7 +28403,7 @@
     </row>
     <row r="47" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="113" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B47" s="113"/>
       <c r="C47" s="113"/>
@@ -28305,7 +28417,7 @@
     </row>
     <row r="48" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="113" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="B48" s="113"/>
       <c r="C48" s="113"/>
@@ -28319,7 +28431,7 @@
     </row>
     <row r="49" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="113" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="B49" s="113"/>
       <c r="C49" s="113"/>
@@ -28333,7 +28445,7 @@
     </row>
     <row r="50" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="113" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B50" s="113"/>
       <c r="C50" s="113"/>
@@ -28362,7 +28474,246 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="11" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="44" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
+    <col min="10" max="10" width="16" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" s="74" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" s="93" t="s">
+        <v>607</v>
+      </c>
+      <c r="B4" s="93" t="s">
+        <v>608</v>
+      </c>
+      <c r="C4" s="93" t="s">
+        <v>609</v>
+      </c>
+      <c r="D4" s="93" t="s">
+        <v>610</v>
+      </c>
+      <c r="E4" s="93" t="s">
+        <v>611</v>
+      </c>
+      <c r="F4" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="G4" s="93" t="s">
+        <v>612</v>
+      </c>
+      <c r="H4" s="93" t="s">
+        <v>613</v>
+      </c>
+      <c r="I4" s="93" t="s">
+        <v>614</v>
+      </c>
+      <c r="J4" s="93" t="s">
+        <v>615</v>
+      </c>
+      <c r="K4" s="93" t="s">
+        <v>616</v>
+      </c>
+      <c r="L4" s="93" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" s="49" t="s">
+        <v>618</v>
+      </c>
+      <c r="B5" s="49" t="s">
+        <v>332</v>
+      </c>
+      <c r="C5" s="49" t="s">
+        <v>468</v>
+      </c>
+      <c r="D5" s="49" t="s">
+        <v>619</v>
+      </c>
+      <c r="E5" s="49" t="s">
+        <v>620</v>
+      </c>
+      <c r="F5" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" s="51">
+        <v>19324742</v>
+      </c>
+      <c r="H5" s="49" t="s">
+        <v>621</v>
+      </c>
+      <c r="I5" s="49" t="s">
+        <v>622</v>
+      </c>
+      <c r="J5" s="51">
+        <v>19324742</v>
+      </c>
+      <c r="K5" s="51">
+        <v>0</v>
+      </c>
+      <c r="L5" s="49" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" s="49" t="s">
+        <v>623</v>
+      </c>
+      <c r="B6" s="49" t="s">
+        <v>332</v>
+      </c>
+      <c r="C6" s="49" t="s">
+        <v>468</v>
+      </c>
+      <c r="D6" s="49" t="s">
+        <v>619</v>
+      </c>
+      <c r="E6" s="49" t="s">
+        <v>620</v>
+      </c>
+      <c r="F6" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" s="51">
+        <v>629862023</v>
+      </c>
+      <c r="H6" s="49" t="s">
+        <v>621</v>
+      </c>
+      <c r="I6" s="49" t="s">
+        <v>624</v>
+      </c>
+      <c r="J6" s="51">
+        <v>629862023</v>
+      </c>
+      <c r="K6" s="51">
+        <v>0</v>
+      </c>
+      <c r="L6" s="49" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="49" t="s">
+        <v>625</v>
+      </c>
+      <c r="B7" s="49" t="s">
+        <v>332</v>
+      </c>
+      <c r="C7" s="49" t="s">
+        <v>468</v>
+      </c>
+      <c r="D7" s="49" t="s">
+        <v>619</v>
+      </c>
+      <c r="E7" s="49" t="s">
+        <v>620</v>
+      </c>
+      <c r="F7" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="51">
+        <v>52769692</v>
+      </c>
+      <c r="H7" s="49" t="s">
+        <v>621</v>
+      </c>
+      <c r="I7" s="49" t="s">
+        <v>626</v>
+      </c>
+      <c r="J7" s="51">
+        <v>52769692</v>
+      </c>
+      <c r="K7" s="51">
+        <v>0</v>
+      </c>
+      <c r="L7" s="49" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="49" t="s">
+        <v>627</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>332</v>
+      </c>
+      <c r="C8" s="49" t="s">
+        <v>468</v>
+      </c>
+      <c r="D8" s="49" t="s">
+        <v>628</v>
+      </c>
+      <c r="E8" s="49" t="s">
+        <v>620</v>
+      </c>
+      <c r="F8" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="51">
+        <v>2709103</v>
+      </c>
+      <c r="H8" s="49" t="s">
+        <v>629</v>
+      </c>
+      <c r="I8" s="49" t="s">
+        <v>630</v>
+      </c>
+      <c r="J8" s="51">
+        <v>2709103</v>
+      </c>
+      <c r="K8" s="51">
+        <v>0</v>
+      </c>
+      <c r="L8" s="49" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="9" spans="6:11" x14ac:dyDescent="0.25">
+      <c r="F9" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G9" s="114">
+        <f>SUM(G5:G8)</f>
+      </c>
+      <c r="J9" s="114">
+        <f>SUM(J5:J8)</f>
+      </c>
+      <c r="K9" s="114">
+        <f>SUM(K5:K8)</f>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -28371,65 +28722,65 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>602</v>
+        <v>631</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="66" t="s">
-        <v>603</v>
+        <v>632</v>
       </c>
       <c r="B3" s="67"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="114" t="s">
-        <v>604</v>
+      <c r="A4" s="115" t="s">
+        <v>633</v>
       </c>
       <c r="B4" s="113" t="s">
-        <v>605</v>
+        <v>634</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="114" t="s">
-        <v>606</v>
+      <c r="A5" s="115" t="s">
+        <v>635</v>
       </c>
       <c r="B5" s="113" t="s">
-        <v>607</v>
+        <v>636</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="114" t="s">
-        <v>608</v>
+      <c r="A6" s="115" t="s">
+        <v>637</v>
       </c>
       <c r="B6" s="113" t="s">
-        <v>609</v>
+        <v>638</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="114" t="s">
-        <v>610</v>
+      <c r="A7" s="115" t="s">
+        <v>639</v>
       </c>
       <c r="B7" s="113" t="s">
-        <v>611</v>
+        <v>640</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="114" t="s">
+      <c r="A8" s="115" t="s">
         <v>39</v>
       </c>
       <c r="B8" s="113" t="s">
-        <v>612</v>
+        <v>641</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="114" t="s">
-        <v>613</v>
+      <c r="A9" s="115" t="s">
+        <v>642</v>
       </c>
       <c r="B9" s="113" t="s">
-        <v>614</v>
+        <v>643</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="114" t="s">
+      <c r="A10" s="115" t="s">
         <v>15</v>
       </c>
       <c r="B10" s="113" t="s">
@@ -28438,156 +28789,164 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="66" t="s">
-        <v>615</v>
+        <v>644</v>
       </c>
       <c r="B11" s="67"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" s="114" t="s">
+      <c r="A12" s="115" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="113" t="s">
-        <v>616</v>
+        <v>645</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" s="114" t="s">
-        <v>617</v>
+      <c r="A13" s="115" t="s">
+        <v>646</v>
       </c>
       <c r="B13" s="113" t="s">
-        <v>618</v>
+        <v>647</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" s="114" t="s">
-        <v>610</v>
+      <c r="A14" s="115" t="s">
+        <v>639</v>
       </c>
       <c r="B14" s="113" t="s">
-        <v>619</v>
+        <v>648</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" s="114" t="s">
-        <v>620</v>
+      <c r="A15" s="115" t="s">
+        <v>649</v>
       </c>
       <c r="B15" s="113" t="s">
-        <v>621</v>
+        <v>650</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" s="114" t="s">
-        <v>613</v>
+      <c r="A16" s="115" t="s">
+        <v>642</v>
       </c>
       <c r="B16" s="113" t="s">
-        <v>622</v>
+        <v>651</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="114" t="s">
-        <v>623</v>
+      <c r="A17" s="115" t="s">
+        <v>652</v>
       </c>
       <c r="B17" s="113" t="s">
-        <v>624</v>
+        <v>653</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="114" t="s">
-        <v>625</v>
+      <c r="A18" s="115" t="s">
+        <v>654</v>
       </c>
       <c r="B18" s="113" t="s">
-        <v>626</v>
+        <v>655</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="114" t="s">
-        <v>627</v>
+      <c r="A19" s="115" t="s">
+        <v>656</v>
       </c>
       <c r="B19" s="113" t="s">
-        <v>628</v>
+        <v>657</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="114" t="s">
+      <c r="A20" s="115" t="s">
+        <v>658</v>
+      </c>
+      <c r="B20" s="113" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="115" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="113" t="s">
+      <c r="B21" s="113" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="66" t="s">
-        <v>629</v>
-      </c>
-      <c r="B21" s="67"/>
-    </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="114" t="s">
-        <v>630</v>
-      </c>
-      <c r="B22" s="113" t="s">
-        <v>631</v>
-      </c>
+      <c r="A22" s="66" t="s">
+        <v>660</v>
+      </c>
+      <c r="B22" s="67"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="114" t="s">
-        <v>632</v>
+      <c r="A23" s="115" t="s">
+        <v>661</v>
       </c>
       <c r="B23" s="113" t="s">
-        <v>633</v>
+        <v>662</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="114" t="s">
-        <v>634</v>
+      <c r="A24" s="115" t="s">
+        <v>663</v>
       </c>
       <c r="B24" s="113" t="s">
-        <v>635</v>
+        <v>664</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="114" t="s">
+      <c r="A25" s="115" t="s">
+        <v>665</v>
+      </c>
+      <c r="B25" s="113" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="115" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="113" t="s">
+      <c r="B26" s="113" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="66" t="s">
-        <v>636</v>
-      </c>
-      <c r="B26" s="67"/>
-    </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="114" t="s">
-        <v>637</v>
-      </c>
-      <c r="B27" s="113" t="s">
-        <v>638</v>
-      </c>
+      <c r="A27" s="66" t="s">
+        <v>667</v>
+      </c>
+      <c r="B27" s="67"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="114" t="s">
-        <v>639</v>
+      <c r="A28" s="115" t="s">
+        <v>668</v>
       </c>
       <c r="B28" s="113" t="s">
-        <v>640</v>
+        <v>669</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="114" t="s">
-        <v>641</v>
+      <c r="A29" s="115" t="s">
+        <v>670</v>
       </c>
       <c r="B29" s="113" t="s">
-        <v>642</v>
+        <v>671</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="114" t="s">
-        <v>643</v>
+      <c r="A30" s="115" t="s">
+        <v>672</v>
       </c>
       <c r="B30" s="113" t="s">
-        <v>644</v>
+        <v>673</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="115" t="s">
+        <v>674</v>
+      </c>
+      <c r="B31" s="113" t="s">
+        <v>675</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Équilibrage : libellé des comptes fonds projet selon leur banque
« ECO fonds projet » au lieu de « BNI fonds projet » pour un fonds projet
Ecobank ; même règle pour les comptes courants et Debt Service.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NEhkcxCB327Mdpf33KqYQU
</commit_message>
<xml_diff>
--- a/Reporting_Hebdo_CIV_30-09-2026.xlsx
+++ b/Reporting_Hebdo_CIV_30-09-2026.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2903" uniqueCount="689">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2903" uniqueCount="690">
   <si>
     <t>Reporting Cash Hebdomadaire – Centralisation Côte d'Ivoire</t>
   </si>
@@ -462,1126 +462,1129 @@
     <t>BACI AGORA</t>
   </si>
   <si>
+    <t>BACI</t>
+  </si>
+  <si>
+    <t>SIB</t>
+  </si>
+  <si>
+    <t>payé par PICI</t>
+  </si>
+  <si>
+    <t>NIVELLEMENT VIA PICI</t>
+  </si>
+  <si>
+    <t>Excédents PICI puis FIRST vers les sociétés en déficit : impôts, cotisations et salaires d'abord, fournisseurs ensuite</t>
+  </si>
+  <si>
+    <t>AUTRES NIVELLEMENTS</t>
+  </si>
+  <si>
+    <t>Virements entre comptes d'une même entité (BNI-RIVIERA courant : sous réserve d'arbitrage)</t>
+  </si>
+  <si>
+    <t>FOURNISSEURS-PROJETS</t>
+  </si>
+  <si>
+    <t>Cash plans : comptes « Dédié paiement CPI » ; SCO AO : BACI-Projet</t>
+  </si>
+  <si>
+    <t>FOURNISSEURS-FGX</t>
+  </si>
+  <si>
+    <t>IMPÔTS</t>
+  </si>
+  <si>
+    <t>ÉCHÉANCES</t>
+  </si>
+  <si>
+    <t>Échéances de prêts FIRST : dépenses de fonctionnement, compte payeur de FIRST</t>
+  </si>
+  <si>
+    <t>AUTRES (ENCAISSEMENTS, DIVERS)</t>
+  </si>
+  <si>
+    <t>ENREGISTREMENTS</t>
+  </si>
+  <si>
+    <t>Hors besoin (droits d'enregistrement, Retenu = N)</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Solde au 30/09/2026</t>
+  </si>
+  <si>
+    <t>Solde théorique fin S1 (11/10/2026)</t>
+  </si>
+  <si>
+    <t>Reste à financer (spot) ou à reporter</t>
+  </si>
+  <si>
+    <t>Virements à passer (modifiables : les nivellements et les soldes ci-dessus se recalculent)</t>
+  </si>
+  <si>
+    <t>Type de nivellement</t>
+  </si>
+  <si>
+    <t>N°</t>
+  </si>
+  <si>
+    <t>Compte source</t>
+  </si>
+  <si>
+    <t>Compte bénéficiaire</t>
+  </si>
+  <si>
+    <t>Montant FCFA</t>
+  </si>
+  <si>
+    <t>Motif</t>
+  </si>
+  <si>
+    <t>RIVIERA PARK – BNI courant</t>
+  </si>
+  <si>
+    <t>RIVIERA PARK – SG</t>
+  </si>
+  <si>
+    <t>Total des virements</t>
+  </si>
+  <si>
+    <t>Comptes (liste de saisie)</t>
+  </si>
+  <si>
+    <t>TERASSON – BNI fonds projet</t>
+  </si>
+  <si>
+    <t>TERASSON – SG</t>
+  </si>
+  <si>
+    <t>TERASSON – ECO</t>
+  </si>
+  <si>
+    <t>PICI – STB</t>
+  </si>
+  <si>
+    <t>PICI – SG</t>
+  </si>
+  <si>
+    <t>PICI – ECO</t>
+  </si>
+  <si>
+    <t>SCI FIRST – STB</t>
+  </si>
+  <si>
+    <t>SCI FIRST – SG</t>
+  </si>
+  <si>
+    <t>RIVIERA PARK – BNI fonds projet</t>
+  </si>
+  <si>
+    <t>SCO AO – BACI Projet</t>
+  </si>
+  <si>
+    <t>SCO AO – BACI courant</t>
+  </si>
+  <si>
+    <t>SCO AO – BOA</t>
+  </si>
+  <si>
+    <t>SCO AO – BACI AGORA</t>
+  </si>
+  <si>
+    <t>SCO AO – ECO</t>
+  </si>
+  <si>
+    <t>IMMONEUF – SG</t>
+  </si>
+  <si>
+    <t>IMMONEUF – BACI</t>
+  </si>
+  <si>
+    <t>IMMONEUF – ECO</t>
+  </si>
+  <si>
+    <t>FINAFRICA – SG</t>
+  </si>
+  <si>
+    <t>FINAFRICA – ECO</t>
+  </si>
+  <si>
+    <t>INFI – SIB</t>
+  </si>
+  <si>
+    <t>ODALYS CI – SG</t>
+  </si>
+  <si>
+    <t>AB CENTER – ECO</t>
+  </si>
+  <si>
+    <t>AB CENTER – SG</t>
+  </si>
+  <si>
+    <t>RHD CI – payé par PICI</t>
+  </si>
+  <si>
+    <t>Détail des flux de fonctionnement (frais de structure) – FCFA</t>
+  </si>
+  <si>
+    <t>Paiement effectué : saisir le montant payé en H (et sa date en I) ; seul le reste à payer (J) alimente le reporting. Paiement non prévu : ajouter une ligne en bas (semaine, entité, nature, libellé, montant négatif, Retenu = O).</t>
+  </si>
+  <si>
+    <t>Nature</t>
+  </si>
+  <si>
+    <t>Fournisseur / libellé</t>
+  </si>
+  <si>
+    <t>Montant €</t>
+  </si>
+  <si>
+    <t>Retenu (O/N)</t>
+  </si>
+  <si>
+    <t>Payé FCFA (saisie)</t>
+  </si>
+  <si>
+    <t>Date de paiement</t>
+  </si>
+  <si>
+    <t>Reste à payer FCFA</t>
+  </si>
+  <si>
+    <t>BURMA</t>
+  </si>
+  <si>
+    <t>O</t>
+  </si>
+  <si>
+    <t>CABINET JEAN-LUC RUELLE</t>
+  </si>
+  <si>
+    <t>CIE</t>
+  </si>
+  <si>
+    <t>DHL</t>
+  </si>
+  <si>
+    <t>FOURNISSEURS DIVERS</t>
+  </si>
+  <si>
+    <t>HORUS TRAD SARL</t>
+  </si>
+  <si>
+    <t>IMPACT</t>
+  </si>
+  <si>
+    <t>JULIE BASSONVILLE</t>
+  </si>
+  <si>
+    <t>LAVIVA</t>
+  </si>
+  <si>
+    <t>LOXEA</t>
+  </si>
+  <si>
+    <t>MISTRAL VOYAGES</t>
+  </si>
+  <si>
+    <t>MTN C“te d'Ivoire</t>
+  </si>
+  <si>
+    <t>NEYALA</t>
+  </si>
+  <si>
+    <t>NOVAGO COTE D'IVOIRE</t>
+  </si>
+  <si>
+    <t>OLEA CI</t>
+  </si>
+  <si>
+    <t>ORANGE CI_TEL MOB</t>
+  </si>
+  <si>
+    <t>SHERPA</t>
+  </si>
+  <si>
+    <t>SODECI</t>
+  </si>
+  <si>
+    <t>TBC</t>
+  </si>
+  <si>
+    <t>Bic</t>
+  </si>
+  <si>
+    <t>Bnc</t>
+  </si>
+  <si>
+    <t>Irc</t>
+  </si>
+  <si>
+    <t>Its</t>
+  </si>
+  <si>
+    <t>PPSSI</t>
+  </si>
+  <si>
+    <t>Tva p/c de tiers</t>
+  </si>
+  <si>
+    <t>Cmu</t>
+  </si>
+  <si>
+    <t>Cnps</t>
+  </si>
+  <si>
+    <t>BOTANICA_BON</t>
+  </si>
+  <si>
+    <t>C2A CONSEIL ASSOCIES</t>
+  </si>
+  <si>
+    <t>ETUDE MAITRE NANOU - NOTAIRE</t>
+  </si>
+  <si>
+    <t>FSSEUR DIVERS</t>
+  </si>
+  <si>
+    <t>MAITRE YAPO KOYO FLORE</t>
+  </si>
+  <si>
+    <t>METALUX</t>
+  </si>
+  <si>
+    <t>MONDON CONSEIL INTERNATIONAL</t>
+  </si>
+  <si>
+    <t>REDEVANCE DIABY</t>
+  </si>
+  <si>
+    <t>SNEF</t>
+  </si>
+  <si>
+    <t>TUNELIER INTERNATIONAL</t>
+  </si>
+  <si>
+    <t>Capital emprunté</t>
+  </si>
+  <si>
+    <t>Stanbic</t>
+  </si>
+  <si>
+    <t>DADIE DIGRA</t>
+  </si>
+  <si>
+    <t>ETUDE DE MAITRE YAPO-KOYO FLORE</t>
+  </si>
+  <si>
+    <t>FORVIS MAZARS</t>
+  </si>
+  <si>
+    <t>CABINET JLR</t>
+  </si>
+  <si>
+    <t>Jetons de présence</t>
+  </si>
+  <si>
+    <t>APPRO CAISSE ELECTRO – Prime transport chantier/frais telecom</t>
+  </si>
+  <si>
+    <t>PKS – gardiennage (gardiennage ancien locaux septembre)</t>
+  </si>
+  <si>
+    <t>PRO SIPEF CI – Trvx de demenagement (trx de descente cablage ancien siege/ validé RIB non transmis)</t>
+  </si>
+  <si>
+    <t>SOFIDEC – CAC (exercice 2025)</t>
+  </si>
+  <si>
+    <t>SYNASPE – numerisation AO (Assistance AO/ Validé / doc bancaire à regulariser)</t>
+  </si>
+  <si>
+    <t>THULIUM – Protocole</t>
+  </si>
+  <si>
+    <t>IVOIRE AGORA SAS – AGORAO KOUMASSI (remis à l'encaissement)</t>
+  </si>
+  <si>
+    <t>AXA</t>
+  </si>
+  <si>
+    <t>CABINET JEAN LUC RUELLE</t>
+  </si>
+  <si>
+    <t>DBL SERVICE &amp; INVEST</t>
+  </si>
+  <si>
+    <t>FSSEURS DIVERS</t>
+  </si>
+  <si>
+    <t>HORUS TRAD</t>
+  </si>
+  <si>
+    <t>KONAN LOAN</t>
+  </si>
+  <si>
+    <t>MAITRE YAPO</t>
+  </si>
+  <si>
+    <t>NAYELA</t>
+  </si>
+  <si>
+    <t>NOVAGO</t>
+  </si>
+  <si>
+    <t>SCOGES CONSEIL</t>
+  </si>
+  <si>
+    <t>CABINET JEAN LUX RUELLE</t>
+  </si>
+  <si>
+    <t>IMPACT DURABLE</t>
+  </si>
+  <si>
+    <t>TEE</t>
+  </si>
+  <si>
+    <t>ADES</t>
+  </si>
+  <si>
+    <t>AILLEURS BUSINESS</t>
+  </si>
+  <si>
+    <t>OFFICE BUREAU</t>
+  </si>
+  <si>
+    <t>Microentreprise</t>
+  </si>
+  <si>
+    <t>MAITRE YAPO-KOYO</t>
+  </si>
+  <si>
+    <t>ENTREPRISE IVOIRIENNE D'AIDE EN ASSAINISSEMENT</t>
+  </si>
+  <si>
+    <t>FOX SECURITE</t>
+  </si>
+  <si>
+    <t>GROUPE LA LAVANDIERE</t>
+  </si>
+  <si>
+    <t>NIMITZ ASC ASSISTANCE SECURITE</t>
+  </si>
+  <si>
+    <t>QUICKNET SERVICE</t>
+  </si>
+  <si>
+    <t>SED SERVICE</t>
+  </si>
+  <si>
+    <t>VISUEL</t>
+  </si>
+  <si>
+    <t>Loyer octobre 2026 – DC/BR</t>
+  </si>
+  <si>
+    <t>Loyer octobre 2026 – ITOCHU CORPORATION SA</t>
+  </si>
+  <si>
+    <t>Loyer octobre 2026 – JESA WEST AFRICA SASU</t>
+  </si>
+  <si>
+    <t>Loyer octobre 2026 – M&amp;H CONSULTING AFRICA SARL</t>
+  </si>
+  <si>
+    <t>Loyer octobre 2026 – SA LOG IVOIRE</t>
+  </si>
+  <si>
+    <t>Loyer octobre 2026 – SBS SOFTWARE IVORY COAST</t>
+  </si>
+  <si>
+    <t>JURIS IMPACT – prestataire juridique</t>
+  </si>
+  <si>
+    <t>LOXEA – location vehicule</t>
+  </si>
+  <si>
+    <t>NEYALA – materiel informatique</t>
+  </si>
+  <si>
+    <t>BETEC-CI – PROJET SAINT PAUL (Suspendu à la demande de Adnane AMAMOU)</t>
+  </si>
+  <si>
+    <t>CMU – cotisation mois et rappel</t>
+  </si>
+  <si>
+    <t>CNPS – declaratioion</t>
+  </si>
+  <si>
+    <t>AGPB – FRAIS GENEAUX BLAISE PASCAL</t>
+  </si>
+  <si>
+    <t>COMETE – MABY (suivant accord de reprise)</t>
+  </si>
+  <si>
+    <t>Salaires</t>
+  </si>
+  <si>
+    <t>IMPACT – Integrateur SAGE</t>
+  </si>
+  <si>
+    <t>IMPOT DGI – Déclaration Septembre</t>
+  </si>
+  <si>
+    <t>PERSONNEL – Salaire Novembre</t>
+  </si>
+  <si>
+    <t>SUD CONSTRUCTION – BCEAO (En attente … relance à effectuer)</t>
+  </si>
+  <si>
+    <t>GENESIS – Integrateur AUTOCARD</t>
+  </si>
+  <si>
+    <t>ORANGE FLOTTE – telephonique</t>
+  </si>
+  <si>
+    <t>CLIM ENERGIE ET SERVICES – PROJET BCEAO ET JACQUES PREV (dernier trimestre 2026)</t>
+  </si>
+  <si>
+    <t>SONAPIE – LOYER</t>
+  </si>
+  <si>
+    <t>TOTAL CI – Carburant</t>
+  </si>
+  <si>
+    <t>Après S5</t>
+  </si>
+  <si>
+    <t>BLUE LIONS (intragroupe)</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>FINANCIERE DUVAL (intragroupe)</t>
+  </si>
+  <si>
+    <t>GROUPE DUVAL (intragroupe)</t>
+  </si>
+  <si>
+    <t>INFISOFTWARE (intragroupe)</t>
+  </si>
+  <si>
+    <t>PELEGRINA FRANCE (intragroupe)</t>
+  </si>
+  <si>
+    <t>SCI FIRST INVEST (intragroupe)</t>
+  </si>
+  <si>
+    <t>Droits d'enregistrement (hors besoin, comme la présentation RCI)</t>
+  </si>
+  <si>
+    <t>PEL FR - ASSISTANCE CONSEIL (intragroupe)</t>
+  </si>
+  <si>
+    <t>PELEGRINA AFRIQUE INVEST (intragroupe)</t>
+  </si>
+  <si>
+    <t>PICI (intragroupe)</t>
+  </si>
+  <si>
+    <t>PEL IMMOBILIER CI CONSTRUCTEUR (intragroupe)</t>
+  </si>
+  <si>
+    <t>FIN AFRICA FR (intragroupe)</t>
+  </si>
+  <si>
+    <t>ASSISTANCE TECHNIQUE PELEGRINA AFR (intragroupe)</t>
+  </si>
+  <si>
+    <t>SAS FINANCIERE DUVAL (intragroupe)</t>
+  </si>
+  <si>
+    <t>SAS GROUPE DUVAL (intragroupe)</t>
+  </si>
+  <si>
+    <t>Loyer octobre 2026 – SIEMENS ENERGY SARL</t>
+  </si>
+  <si>
+    <t>Détail des flux projets &amp; dettes (comptes dédiés)</t>
+  </si>
+  <si>
+    <t>Paiement effectué : saisir le montant payé en FCFA en K (et sa date en L) ; seul le reste à payer (M) alimente le reporting.</t>
+  </si>
+  <si>
+    <t>Compte dédié (clé)</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Libellé</t>
+  </si>
+  <si>
+    <t>Entreprise</t>
+  </si>
+  <si>
+    <t>Montant € HT</t>
+  </si>
+  <si>
+    <t>FON 0009</t>
+  </si>
+  <si>
+    <t>Géomètre</t>
+  </si>
+  <si>
+    <t>KOUAMELAN</t>
+  </si>
+  <si>
+    <t>09 BGTB</t>
+  </si>
+  <si>
+    <t>BCC 0009</t>
+  </si>
+  <si>
+    <t>Autres travaux</t>
+  </si>
+  <si>
+    <t>BCC 0017</t>
+  </si>
+  <si>
+    <t>02 GROS ŒUVRE &amp; INSTALLATION DE CHANTIER</t>
+  </si>
+  <si>
+    <t>07/10/2026</t>
+  </si>
+  <si>
+    <t>BCC 0023</t>
+  </si>
+  <si>
+    <t>07 SERRURERIE</t>
+  </si>
+  <si>
+    <t>BCC 0024</t>
+  </si>
+  <si>
+    <t>08 CFO</t>
+  </si>
+  <si>
+    <t>BCC 0025</t>
+  </si>
+  <si>
+    <t>09A CFA /SSI /GTB</t>
+  </si>
+  <si>
+    <t>HON 0001</t>
+  </si>
+  <si>
+    <t>Architecte</t>
+  </si>
+  <si>
+    <t>ARCHICONCEPT / MAP</t>
+  </si>
+  <si>
+    <t>HON 0002</t>
+  </si>
+  <si>
+    <t>BET / MOE / SSI</t>
+  </si>
+  <si>
+    <t>SCO</t>
+  </si>
+  <si>
+    <t>HON 0005</t>
+  </si>
+  <si>
+    <t>Bureau de contrôle</t>
+  </si>
+  <si>
+    <t>BUREAU VERITAS</t>
+  </si>
+  <si>
+    <t>HON 0006</t>
+  </si>
+  <si>
+    <t>CSPS</t>
+  </si>
+  <si>
+    <t>SOCOTEC</t>
+  </si>
+  <si>
+    <t>HON 0007</t>
+  </si>
+  <si>
+    <t>E&amp;S</t>
+  </si>
+  <si>
+    <t>ANDE / ENVAL / INSUCO / BIOTOPE / IVOIRE HYDROGENE</t>
+  </si>
+  <si>
+    <t>HON 0009</t>
+  </si>
+  <si>
+    <t>Divers honoraires</t>
+  </si>
+  <si>
+    <t>PROJEX / DIPHONE / LUSEO / BET GAURY</t>
+  </si>
+  <si>
+    <t>HON 0010</t>
+  </si>
+  <si>
+    <t>Retenue à la source (prestataires étrangers)</t>
+  </si>
+  <si>
+    <t>AUD 0007</t>
+  </si>
+  <si>
+    <t>Frais Divers</t>
+  </si>
+  <si>
+    <t>YABA &amp; KUMBA / SINTALI / VOLTERE</t>
+  </si>
+  <si>
+    <t>AUD 0012</t>
+  </si>
+  <si>
+    <t>Autres frais financiers (Frais de Due Diligence)</t>
+  </si>
+  <si>
+    <t>DWF/IFC</t>
+  </si>
+  <si>
+    <t>FFI 0001</t>
+  </si>
+  <si>
+    <t>Intérêts sur compte courant</t>
+  </si>
+  <si>
+    <t>FFI 0005</t>
+  </si>
+  <si>
+    <t>Frais Financiers Coupons Invest</t>
+  </si>
+  <si>
+    <t>ATELIER TOPOGRAPHIQUE KOTOKOU / CYGE / SG2T</t>
+  </si>
+  <si>
+    <t>FON 0014</t>
+  </si>
+  <si>
+    <t>Sécurisation du site</t>
+  </si>
+  <si>
+    <t>AIGLE ROYAL / RASCOM / SEG / ECS</t>
+  </si>
+  <si>
+    <t>FON 0018</t>
+  </si>
+  <si>
+    <t>Brche. Eau</t>
+  </si>
+  <si>
+    <t>BCC 0001</t>
+  </si>
+  <si>
+    <t>Démolitions</t>
+  </si>
+  <si>
+    <t>BCC 0002</t>
+  </si>
+  <si>
+    <t>Fondations spéciales</t>
+  </si>
+  <si>
+    <t>BCC 0013</t>
+  </si>
+  <si>
+    <t>1B-VRD - Espaces verts</t>
+  </si>
+  <si>
+    <t>UNISERV</t>
+  </si>
+  <si>
+    <t>BCC 0014</t>
+  </si>
+  <si>
+    <t>2-Gros oeuvre</t>
+  </si>
+  <si>
+    <t>BCC 0015</t>
+  </si>
+  <si>
+    <t>3-Etancheite</t>
+  </si>
+  <si>
+    <t>BCC 0016</t>
+  </si>
+  <si>
+    <t>4A-Charpente metallique</t>
+  </si>
+  <si>
+    <t>4B-Couverture &amp; Bardage</t>
+  </si>
+  <si>
+    <t>BCC 0018</t>
+  </si>
+  <si>
+    <t>5-Menuiseries exterieures</t>
+  </si>
+  <si>
+    <t>BCC 0020</t>
+  </si>
+  <si>
+    <t>7-Serrurerie</t>
+  </si>
+  <si>
+    <t>ZUO / CIA / MAP</t>
+  </si>
+  <si>
+    <t>INSUCO / BRL INGENIERIE/ANDE</t>
+  </si>
+  <si>
+    <t>HON 0008</t>
+  </si>
+  <si>
+    <t>Diagnostic divers</t>
+  </si>
+  <si>
+    <t>AUXO / PROJEX / GSPM / HORECAF / HILLEL</t>
+  </si>
+  <si>
+    <t>AUD 0008</t>
+  </si>
+  <si>
+    <t>Publicité</t>
+  </si>
+  <si>
+    <t>SHERPA/LES ATELIERS COOK IMPRIM</t>
+  </si>
+  <si>
+    <t>FFI 0002</t>
+  </si>
+  <si>
+    <t>Produits financiers</t>
+  </si>
+  <si>
+    <t>03 ETANCHEITE</t>
+  </si>
+  <si>
+    <t>BCC 0034</t>
+  </si>
+  <si>
+    <t>CC ROOFTOP SURELEVATION BAT B</t>
+  </si>
+  <si>
+    <t>FON 0017</t>
+  </si>
+  <si>
+    <t>Brche. Electricité</t>
+  </si>
+  <si>
+    <t>CI ENERGIES</t>
+  </si>
+  <si>
+    <t>8-CFO - Courants forts</t>
+  </si>
+  <si>
+    <t>9-CFA - Courants faibles</t>
+  </si>
+  <si>
+    <t>10-Climatisation &amp; Ventilation</t>
+  </si>
+  <si>
+    <t>11-Plomberie RIA - FC</t>
+  </si>
+  <si>
+    <t>THINKSTEP / YABA &amp; KUMBA / DOUG AND WOLF / CHANAN / REAL CONSULTING / HORECAF / GILLES DEVENDEVILLE</t>
+  </si>
+  <si>
+    <t>AUD 0009</t>
+  </si>
+  <si>
+    <t>Honoraires Juridiques et Fiscaux</t>
+  </si>
+  <si>
+    <t>KSK / MONDON / CHAUVEAU</t>
+  </si>
+  <si>
+    <t>FFI 0003</t>
+  </si>
+  <si>
+    <t>Frais intercalaires</t>
+  </si>
+  <si>
+    <t>FFI 0004</t>
+  </si>
+  <si>
+    <t>Commissions d'engagement</t>
+  </si>
+  <si>
+    <t>Nov. 2026</t>
+  </si>
+  <si>
+    <t>BCC 0008</t>
+  </si>
+  <si>
+    <t>Travaux aménagements preneurs</t>
+  </si>
+  <si>
+    <t>BCC 0026</t>
+  </si>
+  <si>
+    <t>10 CLIMATISATION / VENTILATION / DESENFUMAGE</t>
+  </si>
+  <si>
+    <t>BCC 0027</t>
+  </si>
+  <si>
+    <t>11 PLOMBERIE / RIA</t>
+  </si>
+  <si>
+    <t>BCC 0028</t>
+  </si>
+  <si>
+    <t>12 REVETEMENTS DURS &amp; SOUPLES</t>
+  </si>
+  <si>
+    <t>BCC 0029</t>
+  </si>
+  <si>
+    <t>13 FP &amp; CLOISONNEMENT</t>
+  </si>
+  <si>
+    <t>BCC 0030</t>
+  </si>
+  <si>
+    <t>14 PEINTURE</t>
+  </si>
+  <si>
+    <t>MAZARS/DWF</t>
+  </si>
+  <si>
+    <t>Honoraires de vente</t>
+  </si>
+  <si>
+    <t>HOV 0004</t>
+  </si>
+  <si>
+    <t>Fonds de concours</t>
+  </si>
+  <si>
+    <t>HOV 0005</t>
+  </si>
+  <si>
+    <t>FF&amp;E RT</t>
+  </si>
+  <si>
+    <t>IFC/PROPARCO</t>
+  </si>
+  <si>
+    <t>BCC 0010</t>
+  </si>
+  <si>
+    <t>Exonérations Douanières</t>
+  </si>
+  <si>
+    <t>AUD 0005</t>
+  </si>
+  <si>
+    <t>Dossier Cdac / Et.Marché</t>
+  </si>
+  <si>
+    <t>DEFINA AFRICA / SOLUTION RETAIL / NAWA REAL ESTATE/</t>
+  </si>
+  <si>
+    <t>Remboursement de prêt</t>
+  </si>
+  <si>
+    <t>Commission bancaire – déjà dans les frais financiers des cash plans</t>
+  </si>
+  <si>
+    <t>Bni – déjà dans les frais financiers des cash plans</t>
+  </si>
+  <si>
+    <t>Position de trésorerie CI – soldes bancaires au 30/09/2026</t>
+  </si>
+  <si>
+    <t>Solde FCFA (colonne F, en jaune) modifiable : le reporting et l'équilibrage se recalculent. Colonne J : solde d'origine de la position CI.</t>
+  </si>
+  <si>
+    <t>Banque</t>
+  </si>
+  <si>
+    <t>Compte</t>
+  </si>
+  <si>
+    <t>Bloc du reporting</t>
+  </si>
+  <si>
+    <t>Solde FCFA</t>
+  </si>
+  <si>
+    <t>Solde €</t>
+  </si>
+  <si>
+    <t>Clé</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Solde position CI (origine)</t>
+  </si>
+  <si>
+    <t>Écart (mise à jour)</t>
+  </si>
+  <si>
+    <t>SOCIETE GENERALE</t>
+  </si>
+  <si>
+    <t>SOCIETE GENERALE-PICI</t>
+  </si>
+  <si>
+    <t>Compte de société</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 5</t>
+  </si>
+  <si>
+    <t>STANBIC</t>
+  </si>
+  <si>
+    <t>STANBIC-PICI</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 6</t>
+  </si>
+  <si>
+    <t>ECOBANK</t>
+  </si>
+  <si>
+    <t>ECOBANK-PICI</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 7</t>
+  </si>
+  <si>
+    <t>SOCIETE GENERALE-FIRST</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 9</t>
+  </si>
+  <si>
+    <t>STANBIC-FIRST</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 10</t>
+  </si>
+  <si>
+    <t>SOCIETE GENERALE-TERASSON</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 15</t>
+  </si>
+  <si>
+    <t>ECOBANK -TERASSON</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 16</t>
+  </si>
+  <si>
+    <t>SOCIETE GENERALE-RIVIERA</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 19</t>
+  </si>
+  <si>
+    <t>BNI</t>
+  </si>
+  <si>
+    <t>Affection placement? Ou besoin de fonctionnement</t>
+  </si>
+  <si>
+    <t>Compte dédié</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 20</t>
+  </si>
+  <si>
+    <t>BANK OF AFRICA</t>
+  </si>
+  <si>
+    <t>BANK OF AFRICA-SCO AO</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 23</t>
+  </si>
+  <si>
+    <t>BANQUE ATLANTIQUE</t>
+  </si>
+  <si>
+    <t>BACI-CompteCourant</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 24</t>
+  </si>
+  <si>
+    <t>BACI-Projet</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 25</t>
+  </si>
+  <si>
+    <t>BACI-AGORA</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 26</t>
+  </si>
+  <si>
+    <t>ECOBANK - SCO AO</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 27</t>
+  </si>
+  <si>
+    <t>SOCIETE GENERALE-FINAFRICA</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 29</t>
+  </si>
+  <si>
+    <t>ECOBANK-FINAFRICA</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 30</t>
+  </si>
+  <si>
+    <t>SOCIETE GENERALE-AB CENTER</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 32</t>
+  </si>
+  <si>
+    <t>ECOBANK- AB CENTER</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 33</t>
+  </si>
+  <si>
+    <t>SOCIETE GENERALE-IMMONEUF</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 35</t>
+  </si>
+  <si>
+    <t>ECOBANK-IMMONEUF</t>
+  </si>
+  <si>
+    <t>CIV position, ligne 36</t>
+  </si>
+  <si>
     <t>BACI - IMMONEUF</t>
-  </si>
-  <si>
-    <t>SIB</t>
-  </si>
-  <si>
-    <t>payé par PICI</t>
-  </si>
-  <si>
-    <t>NIVELLEMENT VIA PICI</t>
-  </si>
-  <si>
-    <t>Excédents PICI puis FIRST vers les sociétés en déficit : impôts, cotisations et salaires d'abord, fournisseurs ensuite</t>
-  </si>
-  <si>
-    <t>AUTRES NIVELLEMENTS</t>
-  </si>
-  <si>
-    <t>Virements entre comptes d'une même entité (BNI-RIVIERA courant : sous réserve d'arbitrage)</t>
-  </si>
-  <si>
-    <t>FOURNISSEURS-PROJETS</t>
-  </si>
-  <si>
-    <t>Cash plans : comptes « Dédié paiement CPI » ; SCO AO : BACI-Projet</t>
-  </si>
-  <si>
-    <t>FOURNISSEURS-FGX</t>
-  </si>
-  <si>
-    <t>IMPÔTS</t>
-  </si>
-  <si>
-    <t>ÉCHÉANCES</t>
-  </si>
-  <si>
-    <t>Échéances de prêts FIRST : dépenses de fonctionnement, compte payeur de FIRST</t>
-  </si>
-  <si>
-    <t>AUTRES (ENCAISSEMENTS, DIVERS)</t>
-  </si>
-  <si>
-    <t>ENREGISTREMENTS</t>
-  </si>
-  <si>
-    <t>Hors besoin (droits d'enregistrement, Retenu = N)</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Solde au 30/09/2026</t>
-  </si>
-  <si>
-    <t>Solde théorique fin S1 (11/10/2026)</t>
-  </si>
-  <si>
-    <t>Reste à financer (spot) ou à reporter</t>
-  </si>
-  <si>
-    <t>Virements à passer (modifiables : les nivellements et les soldes ci-dessus se recalculent)</t>
-  </si>
-  <si>
-    <t>Type de nivellement</t>
-  </si>
-  <si>
-    <t>N°</t>
-  </si>
-  <si>
-    <t>Compte source</t>
-  </si>
-  <si>
-    <t>Compte bénéficiaire</t>
-  </si>
-  <si>
-    <t>Montant FCFA</t>
-  </si>
-  <si>
-    <t>Motif</t>
-  </si>
-  <si>
-    <t>RIVIERA PARK – BNI courant</t>
-  </si>
-  <si>
-    <t>RIVIERA PARK – SG</t>
-  </si>
-  <si>
-    <t>Total des virements</t>
-  </si>
-  <si>
-    <t>Comptes (liste de saisie)</t>
-  </si>
-  <si>
-    <t>TERASSON – BNI fonds projet</t>
-  </si>
-  <si>
-    <t>TERASSON – SG</t>
-  </si>
-  <si>
-    <t>TERASSON – ECO</t>
-  </si>
-  <si>
-    <t>PICI – STB</t>
-  </si>
-  <si>
-    <t>PICI – SG</t>
-  </si>
-  <si>
-    <t>PICI – ECO</t>
-  </si>
-  <si>
-    <t>SCI FIRST – STB</t>
-  </si>
-  <si>
-    <t>SCI FIRST – SG</t>
-  </si>
-  <si>
-    <t>RIVIERA PARK – BNI fonds projet</t>
-  </si>
-  <si>
-    <t>SCO AO – BACI Projet</t>
-  </si>
-  <si>
-    <t>SCO AO – BACI courant</t>
-  </si>
-  <si>
-    <t>SCO AO – BOA</t>
-  </si>
-  <si>
-    <t>SCO AO – BACI AGORA</t>
-  </si>
-  <si>
-    <t>SCO AO – ECO</t>
-  </si>
-  <si>
-    <t>IMMONEUF – SG</t>
-  </si>
-  <si>
-    <t>IMMONEUF – BACI - IMMONEUF</t>
-  </si>
-  <si>
-    <t>IMMONEUF – ECO</t>
-  </si>
-  <si>
-    <t>FINAFRICA – SG</t>
-  </si>
-  <si>
-    <t>FINAFRICA – ECO</t>
-  </si>
-  <si>
-    <t>INFI – SIB</t>
-  </si>
-  <si>
-    <t>ODALYS CI – SG</t>
-  </si>
-  <si>
-    <t>AB CENTER – ECO</t>
-  </si>
-  <si>
-    <t>AB CENTER – SG</t>
-  </si>
-  <si>
-    <t>RHD CI – payé par PICI</t>
-  </si>
-  <si>
-    <t>Détail des flux de fonctionnement (frais de structure) – FCFA</t>
-  </si>
-  <si>
-    <t>Paiement effectué : saisir le montant payé en H (et sa date en I) ; seul le reste à payer (J) alimente le reporting. Paiement non prévu : ajouter une ligne en bas (semaine, entité, nature, libellé, montant négatif, Retenu = O).</t>
-  </si>
-  <si>
-    <t>Nature</t>
-  </si>
-  <si>
-    <t>Fournisseur / libellé</t>
-  </si>
-  <si>
-    <t>Montant €</t>
-  </si>
-  <si>
-    <t>Retenu (O/N)</t>
-  </si>
-  <si>
-    <t>Payé FCFA (saisie)</t>
-  </si>
-  <si>
-    <t>Date de paiement</t>
-  </si>
-  <si>
-    <t>Reste à payer FCFA</t>
-  </si>
-  <si>
-    <t>BURMA</t>
-  </si>
-  <si>
-    <t>O</t>
-  </si>
-  <si>
-    <t>CABINET JEAN-LUC RUELLE</t>
-  </si>
-  <si>
-    <t>CIE</t>
-  </si>
-  <si>
-    <t>DHL</t>
-  </si>
-  <si>
-    <t>FOURNISSEURS DIVERS</t>
-  </si>
-  <si>
-    <t>HORUS TRAD SARL</t>
-  </si>
-  <si>
-    <t>IMPACT</t>
-  </si>
-  <si>
-    <t>JULIE BASSONVILLE</t>
-  </si>
-  <si>
-    <t>LAVIVA</t>
-  </si>
-  <si>
-    <t>LOXEA</t>
-  </si>
-  <si>
-    <t>MISTRAL VOYAGES</t>
-  </si>
-  <si>
-    <t>MTN C“te d'Ivoire</t>
-  </si>
-  <si>
-    <t>NEYALA</t>
-  </si>
-  <si>
-    <t>NOVAGO COTE D'IVOIRE</t>
-  </si>
-  <si>
-    <t>OLEA CI</t>
-  </si>
-  <si>
-    <t>ORANGE CI_TEL MOB</t>
-  </si>
-  <si>
-    <t>SHERPA</t>
-  </si>
-  <si>
-    <t>SODECI</t>
-  </si>
-  <si>
-    <t>TBC</t>
-  </si>
-  <si>
-    <t>Bic</t>
-  </si>
-  <si>
-    <t>Bnc</t>
-  </si>
-  <si>
-    <t>Irc</t>
-  </si>
-  <si>
-    <t>Its</t>
-  </si>
-  <si>
-    <t>PPSSI</t>
-  </si>
-  <si>
-    <t>Tva p/c de tiers</t>
-  </si>
-  <si>
-    <t>Cmu</t>
-  </si>
-  <si>
-    <t>Cnps</t>
-  </si>
-  <si>
-    <t>BOTANICA_BON</t>
-  </si>
-  <si>
-    <t>C2A CONSEIL ASSOCIES</t>
-  </si>
-  <si>
-    <t>ETUDE MAITRE NANOU - NOTAIRE</t>
-  </si>
-  <si>
-    <t>FSSEUR DIVERS</t>
-  </si>
-  <si>
-    <t>MAITRE YAPO KOYO FLORE</t>
-  </si>
-  <si>
-    <t>METALUX</t>
-  </si>
-  <si>
-    <t>MONDON CONSEIL INTERNATIONAL</t>
-  </si>
-  <si>
-    <t>REDEVANCE DIABY</t>
-  </si>
-  <si>
-    <t>SNEF</t>
-  </si>
-  <si>
-    <t>TUNELIER INTERNATIONAL</t>
-  </si>
-  <si>
-    <t>Capital emprunté</t>
-  </si>
-  <si>
-    <t>Stanbic</t>
-  </si>
-  <si>
-    <t>DADIE DIGRA</t>
-  </si>
-  <si>
-    <t>ETUDE DE MAITRE YAPO-KOYO FLORE</t>
-  </si>
-  <si>
-    <t>FORVIS MAZARS</t>
-  </si>
-  <si>
-    <t>CABINET JLR</t>
-  </si>
-  <si>
-    <t>Jetons de présence</t>
-  </si>
-  <si>
-    <t>APPRO CAISSE ELECTRO – Prime transport chantier/frais telecom</t>
-  </si>
-  <si>
-    <t>PKS – gardiennage (gardiennage ancien locaux septembre)</t>
-  </si>
-  <si>
-    <t>PRO SIPEF CI – Trvx de demenagement (trx de descente cablage ancien siege/ validé RIB non transmis)</t>
-  </si>
-  <si>
-    <t>SOFIDEC – CAC (exercice 2025)</t>
-  </si>
-  <si>
-    <t>SYNASPE – numerisation AO (Assistance AO/ Validé / doc bancaire à regulariser)</t>
-  </si>
-  <si>
-    <t>THULIUM – Protocole</t>
-  </si>
-  <si>
-    <t>IVOIRE AGORA SAS – AGORAO KOUMASSI (remis à l'encaissement)</t>
-  </si>
-  <si>
-    <t>AXA</t>
-  </si>
-  <si>
-    <t>CABINET JEAN LUC RUELLE</t>
-  </si>
-  <si>
-    <t>DBL SERVICE &amp; INVEST</t>
-  </si>
-  <si>
-    <t>FSSEURS DIVERS</t>
-  </si>
-  <si>
-    <t>HORUS TRAD</t>
-  </si>
-  <si>
-    <t>KONAN LOAN</t>
-  </si>
-  <si>
-    <t>MAITRE YAPO</t>
-  </si>
-  <si>
-    <t>NAYELA</t>
-  </si>
-  <si>
-    <t>NOVAGO</t>
-  </si>
-  <si>
-    <t>SCOGES CONSEIL</t>
-  </si>
-  <si>
-    <t>CABINET JEAN LUX RUELLE</t>
-  </si>
-  <si>
-    <t>IMPACT DURABLE</t>
-  </si>
-  <si>
-    <t>TEE</t>
-  </si>
-  <si>
-    <t>ADES</t>
-  </si>
-  <si>
-    <t>AILLEURS BUSINESS</t>
-  </si>
-  <si>
-    <t>OFFICE BUREAU</t>
-  </si>
-  <si>
-    <t>Microentreprise</t>
-  </si>
-  <si>
-    <t>MAITRE YAPO-KOYO</t>
-  </si>
-  <si>
-    <t>ENTREPRISE IVOIRIENNE D'AIDE EN ASSAINISSEMENT</t>
-  </si>
-  <si>
-    <t>FOX SECURITE</t>
-  </si>
-  <si>
-    <t>GROUPE LA LAVANDIERE</t>
-  </si>
-  <si>
-    <t>NIMITZ ASC ASSISTANCE SECURITE</t>
-  </si>
-  <si>
-    <t>QUICKNET SERVICE</t>
-  </si>
-  <si>
-    <t>SED SERVICE</t>
-  </si>
-  <si>
-    <t>VISUEL</t>
-  </si>
-  <si>
-    <t>Loyer octobre 2026 – DC/BR</t>
-  </si>
-  <si>
-    <t>Loyer octobre 2026 – ITOCHU CORPORATION SA</t>
-  </si>
-  <si>
-    <t>Loyer octobre 2026 – JESA WEST AFRICA SASU</t>
-  </si>
-  <si>
-    <t>Loyer octobre 2026 – M&amp;H CONSULTING AFRICA SARL</t>
-  </si>
-  <si>
-    <t>Loyer octobre 2026 – SA LOG IVOIRE</t>
-  </si>
-  <si>
-    <t>Loyer octobre 2026 – SBS SOFTWARE IVORY COAST</t>
-  </si>
-  <si>
-    <t>JURIS IMPACT – prestataire juridique</t>
-  </si>
-  <si>
-    <t>LOXEA – location vehicule</t>
-  </si>
-  <si>
-    <t>NEYALA – materiel informatique</t>
-  </si>
-  <si>
-    <t>BETEC-CI – PROJET SAINT PAUL (Suspendu à la demande de Adnane AMAMOU)</t>
-  </si>
-  <si>
-    <t>CMU – cotisation mois et rappel</t>
-  </si>
-  <si>
-    <t>CNPS – declaratioion</t>
-  </si>
-  <si>
-    <t>AGPB – FRAIS GENEAUX BLAISE PASCAL</t>
-  </si>
-  <si>
-    <t>COMETE – MABY (suivant accord de reprise)</t>
-  </si>
-  <si>
-    <t>Salaires</t>
-  </si>
-  <si>
-    <t>IMPACT – Integrateur SAGE</t>
-  </si>
-  <si>
-    <t>IMPOT DGI – Déclaration Septembre</t>
-  </si>
-  <si>
-    <t>PERSONNEL – Salaire Novembre</t>
-  </si>
-  <si>
-    <t>SUD CONSTRUCTION – BCEAO (En attente … relance à effectuer)</t>
-  </si>
-  <si>
-    <t>GENESIS – Integrateur AUTOCARD</t>
-  </si>
-  <si>
-    <t>ORANGE FLOTTE – telephonique</t>
-  </si>
-  <si>
-    <t>CLIM ENERGIE ET SERVICES – PROJET BCEAO ET JACQUES PREV (dernier trimestre 2026)</t>
-  </si>
-  <si>
-    <t>SONAPIE – LOYER</t>
-  </si>
-  <si>
-    <t>TOTAL CI – Carburant</t>
-  </si>
-  <si>
-    <t>Après S5</t>
-  </si>
-  <si>
-    <t>BLUE LIONS (intragroupe)</t>
-  </si>
-  <si>
-    <t>N</t>
-  </si>
-  <si>
-    <t>FINANCIERE DUVAL (intragroupe)</t>
-  </si>
-  <si>
-    <t>GROUPE DUVAL (intragroupe)</t>
-  </si>
-  <si>
-    <t>INFISOFTWARE (intragroupe)</t>
-  </si>
-  <si>
-    <t>PELEGRINA FRANCE (intragroupe)</t>
-  </si>
-  <si>
-    <t>SCI FIRST INVEST (intragroupe)</t>
-  </si>
-  <si>
-    <t>Droits d'enregistrement (hors besoin, comme la présentation RCI)</t>
-  </si>
-  <si>
-    <t>PEL FR - ASSISTANCE CONSEIL (intragroupe)</t>
-  </si>
-  <si>
-    <t>PELEGRINA AFRIQUE INVEST (intragroupe)</t>
-  </si>
-  <si>
-    <t>PICI (intragroupe)</t>
-  </si>
-  <si>
-    <t>PEL IMMOBILIER CI CONSTRUCTEUR (intragroupe)</t>
-  </si>
-  <si>
-    <t>FIN AFRICA FR (intragroupe)</t>
-  </si>
-  <si>
-    <t>ASSISTANCE TECHNIQUE PELEGRINA AFR (intragroupe)</t>
-  </si>
-  <si>
-    <t>SAS FINANCIERE DUVAL (intragroupe)</t>
-  </si>
-  <si>
-    <t>SAS GROUPE DUVAL (intragroupe)</t>
-  </si>
-  <si>
-    <t>Loyer octobre 2026 – SIEMENS ENERGY SARL</t>
-  </si>
-  <si>
-    <t>Détail des flux projets &amp; dettes (comptes dédiés)</t>
-  </si>
-  <si>
-    <t>Paiement effectué : saisir le montant payé en FCFA en K (et sa date en L) ; seul le reste à payer (M) alimente le reporting.</t>
-  </si>
-  <si>
-    <t>Compte dédié (clé)</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Libellé</t>
-  </si>
-  <si>
-    <t>Entreprise</t>
-  </si>
-  <si>
-    <t>Montant € HT</t>
-  </si>
-  <si>
-    <t>FON 0009</t>
-  </si>
-  <si>
-    <t>Géomètre</t>
-  </si>
-  <si>
-    <t>KOUAMELAN</t>
-  </si>
-  <si>
-    <t>09 BGTB</t>
-  </si>
-  <si>
-    <t>BCC 0009</t>
-  </si>
-  <si>
-    <t>Autres travaux</t>
-  </si>
-  <si>
-    <t>BCC 0017</t>
-  </si>
-  <si>
-    <t>02 GROS ŒUVRE &amp; INSTALLATION DE CHANTIER</t>
-  </si>
-  <si>
-    <t>07/10/2026</t>
-  </si>
-  <si>
-    <t>BCC 0023</t>
-  </si>
-  <si>
-    <t>07 SERRURERIE</t>
-  </si>
-  <si>
-    <t>BCC 0024</t>
-  </si>
-  <si>
-    <t>08 CFO</t>
-  </si>
-  <si>
-    <t>BCC 0025</t>
-  </si>
-  <si>
-    <t>09A CFA /SSI /GTB</t>
-  </si>
-  <si>
-    <t>HON 0001</t>
-  </si>
-  <si>
-    <t>Architecte</t>
-  </si>
-  <si>
-    <t>ARCHICONCEPT / MAP</t>
-  </si>
-  <si>
-    <t>HON 0002</t>
-  </si>
-  <si>
-    <t>BET / MOE / SSI</t>
-  </si>
-  <si>
-    <t>SCO</t>
-  </si>
-  <si>
-    <t>HON 0005</t>
-  </si>
-  <si>
-    <t>Bureau de contrôle</t>
-  </si>
-  <si>
-    <t>BUREAU VERITAS</t>
-  </si>
-  <si>
-    <t>HON 0006</t>
-  </si>
-  <si>
-    <t>CSPS</t>
-  </si>
-  <si>
-    <t>SOCOTEC</t>
-  </si>
-  <si>
-    <t>HON 0007</t>
-  </si>
-  <si>
-    <t>E&amp;S</t>
-  </si>
-  <si>
-    <t>ANDE / ENVAL / INSUCO / BIOTOPE / IVOIRE HYDROGENE</t>
-  </si>
-  <si>
-    <t>HON 0009</t>
-  </si>
-  <si>
-    <t>Divers honoraires</t>
-  </si>
-  <si>
-    <t>PROJEX / DIPHONE / LUSEO / BET GAURY</t>
-  </si>
-  <si>
-    <t>HON 0010</t>
-  </si>
-  <si>
-    <t>Retenue à la source (prestataires étrangers)</t>
-  </si>
-  <si>
-    <t>AUD 0007</t>
-  </si>
-  <si>
-    <t>Frais Divers</t>
-  </si>
-  <si>
-    <t>YABA &amp; KUMBA / SINTALI / VOLTERE</t>
-  </si>
-  <si>
-    <t>AUD 0012</t>
-  </si>
-  <si>
-    <t>Autres frais financiers (Frais de Due Diligence)</t>
-  </si>
-  <si>
-    <t>DWF/IFC</t>
-  </si>
-  <si>
-    <t>FFI 0001</t>
-  </si>
-  <si>
-    <t>Intérêts sur compte courant</t>
-  </si>
-  <si>
-    <t>FFI 0005</t>
-  </si>
-  <si>
-    <t>Frais Financiers Coupons Invest</t>
-  </si>
-  <si>
-    <t>ATELIER TOPOGRAPHIQUE KOTOKOU / CYGE / SG2T</t>
-  </si>
-  <si>
-    <t>FON 0014</t>
-  </si>
-  <si>
-    <t>Sécurisation du site</t>
-  </si>
-  <si>
-    <t>AIGLE ROYAL / RASCOM / SEG / ECS</t>
-  </si>
-  <si>
-    <t>FON 0018</t>
-  </si>
-  <si>
-    <t>Brche. Eau</t>
-  </si>
-  <si>
-    <t>BCC 0001</t>
-  </si>
-  <si>
-    <t>Démolitions</t>
-  </si>
-  <si>
-    <t>BCC 0002</t>
-  </si>
-  <si>
-    <t>Fondations spéciales</t>
-  </si>
-  <si>
-    <t>BCC 0013</t>
-  </si>
-  <si>
-    <t>1B-VRD - Espaces verts</t>
-  </si>
-  <si>
-    <t>UNISERV</t>
-  </si>
-  <si>
-    <t>BCC 0014</t>
-  </si>
-  <si>
-    <t>2-Gros oeuvre</t>
-  </si>
-  <si>
-    <t>BCC 0015</t>
-  </si>
-  <si>
-    <t>3-Etancheite</t>
-  </si>
-  <si>
-    <t>BCC 0016</t>
-  </si>
-  <si>
-    <t>4A-Charpente metallique</t>
-  </si>
-  <si>
-    <t>4B-Couverture &amp; Bardage</t>
-  </si>
-  <si>
-    <t>BCC 0018</t>
-  </si>
-  <si>
-    <t>5-Menuiseries exterieures</t>
-  </si>
-  <si>
-    <t>BCC 0020</t>
-  </si>
-  <si>
-    <t>7-Serrurerie</t>
-  </si>
-  <si>
-    <t>ZUO / CIA / MAP</t>
-  </si>
-  <si>
-    <t>INSUCO / BRL INGENIERIE/ANDE</t>
-  </si>
-  <si>
-    <t>HON 0008</t>
-  </si>
-  <si>
-    <t>Diagnostic divers</t>
-  </si>
-  <si>
-    <t>AUXO / PROJEX / GSPM / HORECAF / HILLEL</t>
-  </si>
-  <si>
-    <t>AUD 0008</t>
-  </si>
-  <si>
-    <t>Publicité</t>
-  </si>
-  <si>
-    <t>SHERPA/LES ATELIERS COOK IMPRIM</t>
-  </si>
-  <si>
-    <t>FFI 0002</t>
-  </si>
-  <si>
-    <t>Produits financiers</t>
-  </si>
-  <si>
-    <t>03 ETANCHEITE</t>
-  </si>
-  <si>
-    <t>BCC 0034</t>
-  </si>
-  <si>
-    <t>CC ROOFTOP SURELEVATION BAT B</t>
-  </si>
-  <si>
-    <t>FON 0017</t>
-  </si>
-  <si>
-    <t>Brche. Electricité</t>
-  </si>
-  <si>
-    <t>CI ENERGIES</t>
-  </si>
-  <si>
-    <t>8-CFO - Courants forts</t>
-  </si>
-  <si>
-    <t>9-CFA - Courants faibles</t>
-  </si>
-  <si>
-    <t>10-Climatisation &amp; Ventilation</t>
-  </si>
-  <si>
-    <t>11-Plomberie RIA - FC</t>
-  </si>
-  <si>
-    <t>THINKSTEP / YABA &amp; KUMBA / DOUG AND WOLF / CHANAN / REAL CONSULTING / HORECAF / GILLES DEVENDEVILLE</t>
-  </si>
-  <si>
-    <t>AUD 0009</t>
-  </si>
-  <si>
-    <t>Honoraires Juridiques et Fiscaux</t>
-  </si>
-  <si>
-    <t>KSK / MONDON / CHAUVEAU</t>
-  </si>
-  <si>
-    <t>FFI 0003</t>
-  </si>
-  <si>
-    <t>Frais intercalaires</t>
-  </si>
-  <si>
-    <t>FFI 0004</t>
-  </si>
-  <si>
-    <t>Commissions d'engagement</t>
-  </si>
-  <si>
-    <t>Nov. 2026</t>
-  </si>
-  <si>
-    <t>BCC 0008</t>
-  </si>
-  <si>
-    <t>Travaux aménagements preneurs</t>
-  </si>
-  <si>
-    <t>BCC 0026</t>
-  </si>
-  <si>
-    <t>10 CLIMATISATION / VENTILATION / DESENFUMAGE</t>
-  </si>
-  <si>
-    <t>BCC 0027</t>
-  </si>
-  <si>
-    <t>11 PLOMBERIE / RIA</t>
-  </si>
-  <si>
-    <t>BCC 0028</t>
-  </si>
-  <si>
-    <t>12 REVETEMENTS DURS &amp; SOUPLES</t>
-  </si>
-  <si>
-    <t>BCC 0029</t>
-  </si>
-  <si>
-    <t>13 FP &amp; CLOISONNEMENT</t>
-  </si>
-  <si>
-    <t>BCC 0030</t>
-  </si>
-  <si>
-    <t>14 PEINTURE</t>
-  </si>
-  <si>
-    <t>MAZARS/DWF</t>
-  </si>
-  <si>
-    <t>Honoraires de vente</t>
-  </si>
-  <si>
-    <t>HOV 0004</t>
-  </si>
-  <si>
-    <t>Fonds de concours</t>
-  </si>
-  <si>
-    <t>HOV 0005</t>
-  </si>
-  <si>
-    <t>FF&amp;E RT</t>
-  </si>
-  <si>
-    <t>IFC/PROPARCO</t>
-  </si>
-  <si>
-    <t>BCC 0010</t>
-  </si>
-  <si>
-    <t>Exonérations Douanières</t>
-  </si>
-  <si>
-    <t>AUD 0005</t>
-  </si>
-  <si>
-    <t>Dossier Cdac / Et.Marché</t>
-  </si>
-  <si>
-    <t>DEFINA AFRICA / SOLUTION RETAIL / NAWA REAL ESTATE/</t>
-  </si>
-  <si>
-    <t>Remboursement de prêt</t>
-  </si>
-  <si>
-    <t>Commission bancaire – déjà dans les frais financiers des cash plans</t>
-  </si>
-  <si>
-    <t>Bni – déjà dans les frais financiers des cash plans</t>
-  </si>
-  <si>
-    <t>Position de trésorerie CI – soldes bancaires au 30/09/2026</t>
-  </si>
-  <si>
-    <t>Solde FCFA (colonne F, en jaune) modifiable : le reporting et l'équilibrage se recalculent. Colonne J : solde d'origine de la position CI.</t>
-  </si>
-  <si>
-    <t>Banque</t>
-  </si>
-  <si>
-    <t>Compte</t>
-  </si>
-  <si>
-    <t>Bloc du reporting</t>
-  </si>
-  <si>
-    <t>Solde FCFA</t>
-  </si>
-  <si>
-    <t>Solde €</t>
-  </si>
-  <si>
-    <t>Clé</t>
-  </si>
-  <si>
-    <t>Source</t>
-  </si>
-  <si>
-    <t>Solde position CI (origine)</t>
-  </si>
-  <si>
-    <t>Écart (mise à jour)</t>
-  </si>
-  <si>
-    <t>SOCIETE GENERALE</t>
-  </si>
-  <si>
-    <t>SOCIETE GENERALE-PICI</t>
-  </si>
-  <si>
-    <t>Compte de société</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 5</t>
-  </si>
-  <si>
-    <t>STANBIC</t>
-  </si>
-  <si>
-    <t>STANBIC-PICI</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 6</t>
-  </si>
-  <si>
-    <t>ECOBANK</t>
-  </si>
-  <si>
-    <t>ECOBANK-PICI</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 7</t>
-  </si>
-  <si>
-    <t>SOCIETE GENERALE-FIRST</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 9</t>
-  </si>
-  <si>
-    <t>STANBIC-FIRST</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 10</t>
-  </si>
-  <si>
-    <t>SOCIETE GENERALE-TERASSON</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 15</t>
-  </si>
-  <si>
-    <t>ECOBANK -TERASSON</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 16</t>
-  </si>
-  <si>
-    <t>SOCIETE GENERALE-RIVIERA</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 19</t>
-  </si>
-  <si>
-    <t>BNI</t>
-  </si>
-  <si>
-    <t>Affection placement? Ou besoin de fonctionnement</t>
-  </si>
-  <si>
-    <t>Compte dédié</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 20</t>
-  </si>
-  <si>
-    <t>BANK OF AFRICA</t>
-  </si>
-  <si>
-    <t>BANK OF AFRICA-SCO AO</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 23</t>
-  </si>
-  <si>
-    <t>BANQUE ATLANTIQUE</t>
-  </si>
-  <si>
-    <t>BACI-CompteCourant</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 24</t>
-  </si>
-  <si>
-    <t>BACI-Projet</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 25</t>
-  </si>
-  <si>
-    <t>BACI-AGORA</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 26</t>
-  </si>
-  <si>
-    <t>ECOBANK - SCO AO</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 27</t>
-  </si>
-  <si>
-    <t>SOCIETE GENERALE-FINAFRICA</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 29</t>
-  </si>
-  <si>
-    <t>ECOBANK-FINAFRICA</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 30</t>
-  </si>
-  <si>
-    <t>SOCIETE GENERALE-AB CENTER</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 32</t>
-  </si>
-  <si>
-    <t>ECOBANK- AB CENTER</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 33</t>
-  </si>
-  <si>
-    <t>SOCIETE GENERALE-IMMONEUF</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 35</t>
-  </si>
-  <si>
-    <t>ECOBANK-IMMONEUF</t>
-  </si>
-  <si>
-    <t>CIV position, ligne 36</t>
   </si>
   <si>
     <t>CIV position, ligne 37</t>
@@ -10514,7 +10517,7 @@
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"IMMONEUF – SG")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"IMMONEUF – SG")</f>
       </c>
       <c r="S7" s="78">
-        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"IMMONEUF – BACI - IMMONEUF")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"IMMONEUF – BACI - IMMONEUF")</f>
+        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"IMMONEUF – BACI")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"IMMONEUF – BACI")</f>
       </c>
       <c r="T7" s="78">
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$E$25:$E$55,"IMMONEUF – ECO")-SUMIFS($H$25:$H$55,$A$25:$A$55,"NIVELLEMENT VIA PICI",$C$25:$C$55,"IMMONEUF – ECO")</f>
@@ -10600,7 +10603,7 @@
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"IMMONEUF – SG")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"IMMONEUF – SG")</f>
       </c>
       <c r="S8" s="78">
-        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"IMMONEUF – BACI - IMMONEUF")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"IMMONEUF – BACI - IMMONEUF")</f>
+        <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"IMMONEUF – BACI")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"IMMONEUF – BACI")</f>
       </c>
       <c r="T8" s="78">
         <f>SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$E$25:$E$55,"IMMONEUF – ECO")-SUMIFS($H$25:$H$55,$A$25:$A$55,"AUTRES NIVELLEMENTS",$C$25:$C$55,"IMMONEUF – ECO")</f>
@@ -27377,7 +27380,7 @@
         <v>15</v>
       </c>
       <c r="C25" s="49" t="s">
-        <v>147</v>
+        <v>521</v>
       </c>
       <c r="D25" s="49" t="s">
         <v>27</v>
@@ -27395,7 +27398,7 @@
         <v>53</v>
       </c>
       <c r="I25" s="49" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="J25" s="51">
         <v>58000</v>
@@ -27412,7 +27415,7 @@
         <v>148</v>
       </c>
       <c r="C26" s="49" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="D26" s="49" t="s">
         <v>27</v>
@@ -27430,7 +27433,7 @@
         <v>57</v>
       </c>
       <c r="I26" s="49" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="J26" s="51">
         <v>2751880</v>
@@ -27447,7 +27450,7 @@
         <v>473</v>
       </c>
       <c r="C27" s="49" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="D27" s="49" t="s">
         <v>27</v>
@@ -27465,7 +27468,7 @@
         <v>59</v>
       </c>
       <c r="I27" s="49" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="J27" s="51">
         <v>6062002</v>
@@ -27485,7 +27488,7 @@
         <v>68</v>
       </c>
       <c r="D28" s="49" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E28" s="49" t="s">
         <v>495</v>
@@ -27500,7 +27503,7 @@
         <v>67</v>
       </c>
       <c r="I28" s="49" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="J28" s="51">
         <v>2643139493</v>
@@ -27520,7 +27523,7 @@
         <v>71</v>
       </c>
       <c r="D29" s="49" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E29" s="49" t="s">
         <v>495</v>
@@ -27535,7 +27538,7 @@
         <v>70</v>
       </c>
       <c r="I29" s="49" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="J29" s="51">
         <v>1481904490</v>
@@ -27570,7 +27573,7 @@
         <v>72</v>
       </c>
       <c r="I30" s="49" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="J30" s="51">
         <v>76268390</v>
@@ -27581,7 +27584,7 @@
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="104" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F31" s="105">
         <f>SUM(F5:F30)</f>
@@ -27592,7 +27595,7 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -27609,7 +27612,7 @@
         <v>79</v>
       </c>
       <c r="E35" s="98" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F35" s="99">
         <v>350727089</v>
@@ -27621,7 +27624,7 @@
         <v>15</v>
       </c>
       <c r="I35" s="98" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="J35" s="98">
         <v>350727089</v>
@@ -27641,7 +27644,7 @@
         <v>79</v>
       </c>
       <c r="E36" s="98" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F36" s="99">
         <v>42500000</v>
@@ -27653,7 +27656,7 @@
         <v>15</v>
       </c>
       <c r="I36" s="98" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="J36" s="98">
         <v>42500000</v>
@@ -27673,7 +27676,7 @@
         <v>79</v>
       </c>
       <c r="E37" s="98" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F37" s="99">
         <v>26289357</v>
@@ -27685,7 +27688,7 @@
         <v>15</v>
       </c>
       <c r="I37" s="98" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="J37" s="98">
         <v>26289357</v>
@@ -27705,7 +27708,7 @@
         <v>79</v>
       </c>
       <c r="E38" s="98" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F38" s="99">
         <v>0</v>
@@ -27717,7 +27720,7 @@
         <v>15</v>
       </c>
       <c r="I38" s="98" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="J38" s="98">
         <v>0</v>
@@ -27737,7 +27740,7 @@
         <v>79</v>
       </c>
       <c r="E39" s="98" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F39" s="99">
         <v>776110097</v>
@@ -27749,7 +27752,7 @@
         <v>15</v>
       </c>
       <c r="I39" s="98" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="J39" s="98">
         <v>776110097</v>
@@ -27757,7 +27760,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="106" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F40" s="107">
         <f>SUM(F35:F39)</f>
@@ -27783,34 +27786,34 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="93" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B4" s="93" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C4" s="93" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D4" s="93" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E4" s="93" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="49" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B5" s="51">
         <f>'Reporting Hebdo'!M52</f>
@@ -27822,12 +27825,12 @@
         <f>B5-C5</f>
       </c>
       <c r="E5" s="49" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -27835,16 +27838,16 @@
         <v>97</v>
       </c>
       <c r="B8" s="93" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="C8" s="93" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="D8" s="93" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E8" s="93" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -27861,7 +27864,7 @@
         <f>B9-C9</f>
       </c>
       <c r="E9" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -27878,7 +27881,7 @@
         <f>B10-C10</f>
       </c>
       <c r="E10" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -27895,7 +27898,7 @@
         <f>B11-C11</f>
       </c>
       <c r="E11" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -27912,7 +27915,7 @@
         <f>B12-C12</f>
       </c>
       <c r="E12" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -27929,7 +27932,7 @@
         <f>B13-C13</f>
       </c>
       <c r="E13" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -27946,7 +27949,7 @@
         <f>B14-C14</f>
       </c>
       <c r="E14" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -27963,7 +27966,7 @@
         <f>B15-C15</f>
       </c>
       <c r="E15" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -27980,7 +27983,7 @@
         <f>B16-C16</f>
       </c>
       <c r="E16" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -27997,26 +28000,26 @@
         <f>B17-C17</f>
       </c>
       <c r="E17" s="49" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="93" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B20" s="93" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="C20" s="93" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="D20" s="93" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E20" s="93" t="s">
         <v>470</v>
@@ -28024,7 +28027,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="49" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B21" s="51">
         <f>-SUMIFS('Détail projets &amp; dettes'!$H$5:$H$500,'Détail projets &amp; dettes'!$C$5:$C$500,"RIVIERA",'Détail projets &amp; dettes'!$J$5:$J$500,"O",'Détail projets &amp; dettes'!$A$5:$A$500,"S*")</f>
@@ -28036,12 +28039,12 @@
         <f>B21-C21</f>
       </c>
       <c r="E21" s="49" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="49" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B22" s="51">
         <f>-SUMIFS('Détail projets &amp; dettes'!$H$5:$H$500,'Détail projets &amp; dettes'!$C$5:$C$500,"TERASSON",'Détail projets &amp; dettes'!$J$5:$J$500,"O",'Détail projets &amp; dettes'!$A$5:$A$500,"S*")</f>
@@ -28053,34 +28056,34 @@
         <f>B22-C22</f>
       </c>
       <c r="E22" s="49" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="93" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B25" s="93" t="s">
         <v>172</v>
       </c>
       <c r="C25" s="93" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D25" s="93" t="s">
         <v>15</v>
       </c>
       <c r="E25" s="93" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="49" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B26" s="51">
         <v>-13254203304</v>
@@ -28092,12 +28095,12 @@
         <v>15</v>
       </c>
       <c r="E26" s="49" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="49" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B27" s="51">
         <v>-1715342550</v>
@@ -28109,12 +28112,12 @@
         <v>15</v>
       </c>
       <c r="E27" s="49" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="49" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="B28" s="51">
         <v>6113285</v>
@@ -28126,12 +28129,12 @@
         <v>15</v>
       </c>
       <c r="E28" s="49" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="49" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="B29" s="51">
         <v>-220402934</v>
@@ -28143,22 +28146,22 @@
         <v>15</v>
       </c>
       <c r="E29" s="49" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" s="89" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" s="89" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
     </row>
   </sheetData>
@@ -28181,12 +28184,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -28194,31 +28197,31 @@
         <v>97</v>
       </c>
       <c r="B4" s="93" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="C4" s="93" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D4" s="93" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E4" s="93" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="F4" s="93" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="G4" s="93" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="H4" s="93" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="I4" s="93" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="J4" s="93" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -28250,7 +28253,7 @@
         <v>-704.66556</v>
       </c>
       <c r="J5" s="111" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -28282,7 +28285,7 @@
         <v>-5.684341886080802e-14</v>
       </c>
       <c r="J6" s="111" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -28314,7 +28317,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="111" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -28346,7 +28349,7 @@
         <v>1.4210854715202004e-14</v>
       </c>
       <c r="J8" s="111" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -28372,7 +28375,7 @@
         <v>-29.545979600000003</v>
       </c>
       <c r="J9" s="111" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -28404,7 +28407,7 @@
         <v>2.842170943040401e-14</v>
       </c>
       <c r="J10" s="111" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -28436,7 +28439,7 @@
         <v>0</v>
       </c>
       <c r="J11" s="111" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -28468,7 +28471,7 @@
         <v>-1.4210854715202004e-14</v>
       </c>
       <c r="J12" s="111" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -28494,7 +28497,7 @@
         <v>2.75188</v>
       </c>
       <c r="J13" s="111" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -28526,7 +28529,7 @@
         <v>-1.7763568394002505e-15</v>
       </c>
       <c r="J14" s="111" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -28558,7 +28561,7 @@
         <v>-1.4210854715202004e-14</v>
       </c>
       <c r="J15" s="111" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -28595,29 +28598,29 @@
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="93" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="B19" s="93" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="C19" s="93" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="D19" s="93" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E19" s="93" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="49" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="B20" s="110">
         <v>244.99626199999997</v>
@@ -28629,12 +28632,12 @@
         <v>0</v>
       </c>
       <c r="E20" s="49" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="49" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="B21" s="110">
         <v>637.405803</v>
@@ -28646,12 +28649,12 @@
         <v>0</v>
       </c>
       <c r="E21" s="49" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="49" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="B22" s="110">
         <v>152.070689</v>
@@ -28663,7 +28666,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="49" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -28680,12 +28683,12 @@
         <v>0</v>
       </c>
       <c r="E23" s="49" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="49" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="B24" s="110">
         <v>448.13497721294</v>
@@ -28697,12 +28700,12 @@
         <v>0</v>
       </c>
       <c r="E24" s="49" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="49" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="B25" s="110">
         <v>129.56826523</v>
@@ -28714,12 +28717,12 @@
         <v>-2.842170943040401e-14</v>
       </c>
       <c r="E25" s="49" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="49" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B26" s="110">
         <v>0</v>
@@ -28731,29 +28734,29 @@
         <v>178.0456286</v>
       </c>
       <c r="E26" s="49" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="93" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="B29" s="93" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="C29" s="93" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D29" s="93" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="E29" s="93" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -28770,12 +28773,12 @@
         <v>4.547473508864641e-13</v>
       </c>
       <c r="E30" s="54" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="49" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="B31" s="110">
         <v>91.2699500964329</v>
@@ -28787,12 +28790,12 @@
         <v>0</v>
       </c>
       <c r="E31" s="49" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="49" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B32" s="110">
         <v>1976.5850833750312</v>
@@ -28804,12 +28807,12 @@
         <v>0</v>
       </c>
       <c r="E32" s="49" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="49" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B33" s="110">
         <v>1267.9055957833798</v>
@@ -28821,12 +28824,12 @@
         <v>2.2737367544323206e-13</v>
       </c>
       <c r="E33" s="49" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="49" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B34" s="110">
         <v>455.07613148087546</v>
@@ -28838,12 +28841,12 @@
         <v>-1.1368683772161603e-13</v>
       </c>
       <c r="E34" s="49" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="49" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B35" s="110">
         <v>2643.139493</v>
@@ -28855,7 +28858,7 @@
         <v>0</v>
       </c>
       <c r="E35" s="49" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -28872,12 +28875,12 @@
         <v>-704.6655599999999</v>
       </c>
       <c r="E36" s="54" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="49" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="B37" s="110">
         <v>116.22847414168119</v>
@@ -28889,12 +28892,12 @@
         <v>1.4210854715202004e-14</v>
       </c>
       <c r="E37" s="49" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="49" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="B38" s="110">
         <v>2197.7624460785723</v>
@@ -28906,12 +28909,12 @@
         <v>0</v>
       </c>
       <c r="E38" s="49" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="49" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="B39" s="110">
         <v>490.0631747136942</v>
@@ -28923,12 +28926,12 @@
         <v>0</v>
       </c>
       <c r="E39" s="49" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="49" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="B40" s="110">
         <v>1238.4883764116369</v>
@@ -28940,12 +28943,12 @@
         <v>-2.2737367544323206e-13</v>
       </c>
       <c r="E40" s="49" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="49" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="B41" s="110">
         <v>1481.90449</v>
@@ -28957,17 +28960,17 @@
         <v>0</v>
       </c>
       <c r="E41" s="49" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
     </row>
     <row r="44" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="113" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="B44" s="113"/>
       <c r="C44" s="113"/>
@@ -28981,7 +28984,7 @@
     </row>
     <row r="45" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="113" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="B45" s="113"/>
       <c r="C45" s="113"/>
@@ -28995,7 +28998,7 @@
     </row>
     <row r="46" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="113" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B46" s="113"/>
       <c r="C46" s="113"/>
@@ -29009,7 +29012,7 @@
     </row>
     <row r="47" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="113" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="B47" s="113"/>
       <c r="C47" s="113"/>
@@ -29023,7 +29026,7 @@
     </row>
     <row r="48" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="113" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="B48" s="113"/>
       <c r="C48" s="113"/>
@@ -29037,7 +29040,7 @@
     </row>
     <row r="49" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="113" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="B49" s="113"/>
       <c r="C49" s="113"/>
@@ -29051,7 +29054,7 @@
     </row>
     <row r="50" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="113" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="B50" s="113"/>
       <c r="C50" s="113"/>
@@ -29099,55 +29102,55 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="74" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="93" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="B4" s="93" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="C4" s="93" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="D4" s="93" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="E4" s="93" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="F4" s="93" t="s">
         <v>97</v>
       </c>
       <c r="G4" s="93" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="H4" s="93" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="I4" s="93" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="J4" s="93" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="K4" s="93" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="L4" s="93" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="49" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="B5" s="49" t="s">
         <v>345</v>
@@ -29156,10 +29159,10 @@
         <v>481</v>
       </c>
       <c r="D5" s="49" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E5" s="49" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F5" s="49" t="s">
         <v>33</v>
@@ -29168,10 +29171,10 @@
         <v>19324742</v>
       </c>
       <c r="H5" s="49" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="I5" s="49" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="J5" s="51">
         <v>19324742</v>
@@ -29185,7 +29188,7 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="49" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="B6" s="49" t="s">
         <v>345</v>
@@ -29194,10 +29197,10 @@
         <v>481</v>
       </c>
       <c r="D6" s="49" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E6" s="49" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F6" s="49" t="s">
         <v>33</v>
@@ -29206,10 +29209,10 @@
         <v>629862023</v>
       </c>
       <c r="H6" s="49" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="I6" s="49" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="J6" s="51">
         <v>629862023</v>
@@ -29223,7 +29226,7 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="49" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="B7" s="49" t="s">
         <v>345</v>
@@ -29232,10 +29235,10 @@
         <v>481</v>
       </c>
       <c r="D7" s="49" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E7" s="49" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F7" s="49" t="s">
         <v>33</v>
@@ -29244,10 +29247,10 @@
         <v>52769692</v>
       </c>
       <c r="H7" s="49" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="I7" s="49" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="J7" s="51">
         <v>52769692</v>
@@ -29261,7 +29264,7 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="49" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="B8" s="49" t="s">
         <v>345</v>
@@ -29270,10 +29273,10 @@
         <v>481</v>
       </c>
       <c r="D8" s="49" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E8" s="49" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F8" s="49" t="s">
         <v>33</v>
@@ -29282,10 +29285,10 @@
         <v>2709103</v>
       </c>
       <c r="H8" s="49" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="I8" s="49" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="J8" s="51">
         <v>2709103</v>
@@ -29328,45 +29331,45 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="66" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B3" s="67"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="115" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B4" s="113" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="115" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="B5" s="113" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="115" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="B6" s="113" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="115" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B7" s="113" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -29374,15 +29377,15 @@
         <v>39</v>
       </c>
       <c r="B8" s="113" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="115" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B9" s="113" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -29395,7 +29398,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="66" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="B11" s="67"/>
     </row>
@@ -29404,71 +29407,71 @@
         <v>3</v>
       </c>
       <c r="B12" s="113" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="115" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B13" s="113" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="115" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="B14" s="113" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="115" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="B15" s="113" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="115" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="B16" s="113" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="115" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="B17" s="113" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="115" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B18" s="113" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="115" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="B19" s="113" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="115" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B20" s="113" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -29481,32 +29484,32 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="66" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B22" s="67"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="115" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="B23" s="113" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="115" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="B24" s="113" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="115" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="B25" s="113" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -29519,40 +29522,40 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="66" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B27" s="67"/>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="115" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="B28" s="113" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="115" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="B29" s="113" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="115" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="B30" s="113" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="115" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="B31" s="113" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
     </row>
   </sheetData>

</xml_diff>